<commit_message>
AnhDXH up last CL target
</commit_message>
<xml_diff>
--- a/Study_CL.xlsx
+++ b/Study_CL.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="10"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Knowhow" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="#6" sheetId="9" r:id="rId9"/>
     <sheet name="#7" sheetId="10" r:id="rId10"/>
     <sheet name="#8" sheetId="11" r:id="rId11"/>
+    <sheet name="#14" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="503">
   <si>
     <t>No.</t>
   </si>
@@ -1640,9 +1641,6 @@
   </si>
   <si>
     <t>Gmock</t>
-  </si>
-  <si>
-    <t>Các Segment trong C++</t>
   </si>
   <si>
     <t>#8</t>
@@ -3632,6 +3630,276 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>#14</t>
+  </si>
+  <si>
+    <t>Các thuật toán sort phổ biến trong C++. Triển khai minh họa.</t>
+  </si>
+  <si>
+    <t>https://chatgpt.com/share/690b291c-d088-8002-b37a-10bb5da410ce</t>
+  </si>
+  <si>
+    <t>What is the difference between ++i and i++</t>
+  </si>
+  <si>
+    <t>Các Segment trong C++ ( Data Segment)</t>
+  </si>
+  <si>
+    <t>RAII là gì (Resource Acquisition Is Initialization)</t>
+  </si>
+  <si>
+    <t>Điều gì xảy ra khi double delete, cách phòng tránh ?</t>
+  </si>
+  <si>
+    <t>Cách phòng tránh</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Khi delete 1 con trỏ, nó trở thành </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dangling pointer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Nếu delete 1 con trỏ 2 lần , sẽ xảy ra hiện tượng "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Undefined Behavior</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" vì </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>hệ thống quản lý bộ nhớ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> không cho phép giải phóng 1 con trỏ đã giải phóng rồi</t>
+    </r>
+  </si>
+  <si>
+    <t>Cấp phát động trong C và C++</t>
+  </si>
+  <si>
+    <t>Cách 1</t>
+  </si>
+  <si>
+    <t>Cách 2</t>
+  </si>
+  <si>
+    <t>Sau khi delete con trỏ, set nó về nullptr, vì xóa nullptr là hợp lệ</t>
+  </si>
+  <si>
+    <t>Sử dụng unique pointer</t>
+  </si>
+  <si>
+    <t>* Rất khó để phát hiện 1 biến con trỏ có đang là dangling pointer không, vì vậy, hãy chủ động phòng tránh bằng cách set nullptr hoặc dùng unique ptr luôn</t>
+  </si>
+  <si>
+    <t>#15</t>
+  </si>
+  <si>
+    <t>#16</t>
+  </si>
+  <si>
+    <t>Ôn lại OOP</t>
+  </si>
+  <si>
+    <t>Sự khác biệt giữa virtual, pure virtual và override</t>
+  </si>
+  <si>
+    <t>What happens if a base class destructor is not virtual?</t>
+  </si>
+  <si>
+    <t>Can constructors be virtual?</t>
+  </si>
+  <si>
+    <t>What is slicing in C++?</t>
+  </si>
+  <si>
+    <t>#17</t>
+  </si>
+  <si>
+    <t>C++ hiện đại</t>
+  </si>
+  <si>
+    <t>Phân biệt rvalue và lvalue ? What are rvalue references (&amp;&amp;) used for?</t>
+  </si>
+  <si>
+    <t>What is the difference between emplace_back() and push_back()?</t>
+  </si>
+  <si>
+    <t>What is a lambda function in C++?</t>
+  </si>
+  <si>
+    <t>#18</t>
+  </si>
+  <si>
+    <t>Containers (vector, list, map, set, queue, stack, …)</t>
+  </si>
+  <si>
+    <t>Algorithms (sort(), find(), count(), max_element(), …)</t>
+  </si>
+  <si>
+    <t>STL (Standard Template Library) &amp; Algorithms</t>
+  </si>
+  <si>
+    <t>Khác biệt giữa compile-time polymorphism ( đa hình lúc biên dịch) và runtime polymorphism ( đa hình lúc chạy).</t>
+  </si>
+  <si>
+    <t>Over loading, Over riding</t>
+  </si>
+  <si>
+    <t>#19</t>
+  </si>
+  <si>
+    <t>Làm thế nào để tránh Memory leak ( và các tool tránh)</t>
+  </si>
+  <si>
+    <t>https://chatgpt.com/share/690b28bd-0994-8002-8476-6d34821ba602</t>
+  </si>
+  <si>
+    <t>#20</t>
+  </si>
+  <si>
+    <t>#21</t>
+  </si>
+  <si>
+    <t>#23</t>
+  </si>
+  <si>
+    <t>https://chatgpt.com/share/690b2878-1980-8002-a972-852d53b05b6d</t>
+  </si>
+  <si>
+    <t>#24</t>
+  </si>
+  <si>
+    <t>Design Pattern phổ biến</t>
+  </si>
+  <si>
+    <t>What is the purpose of std::move()?, Move constructor và move assignment operation ? move semantics ? perfect forwarding ?</t>
+  </si>
+  <si>
+    <t>Khi bạn phải xử lý bug khó tái hiện (intermittent bug) trong hệ thống multi-threaded, bạn sẽ làm gì?</t>
+  </si>
+  <si>
+    <t>https://chatgpt.com/share/690b2849-8930-8002-8e74-c83657de06f5</t>
+  </si>
+  <si>
+    <t>Xem thêm</t>
+  </si>
+  <si>
+    <t>#n</t>
+  </si>
+  <si>
+    <t>Access modifiers : Private, Public, Protected</t>
+  </si>
+  <si>
+    <t>#25</t>
+  </si>
+  <si>
+    <t>Module mày làm gì (CSRC, OpenAPI) ? Đóng vai trò thế nào trong dự án, triển khai theo mô hình nào ?</t>
+  </si>
+  <si>
+    <t>#26</t>
+  </si>
+  <si>
+    <t>Struct vs Union</t>
+  </si>
+  <si>
+    <t>Function pointer</t>
+  </si>
+  <si>
+    <t>Quản lý memory như nào cho hiệu quả</t>
+  </si>
+  <si>
+    <t>Khác nhau giữa C và C++, Data alignment and padding of struct/class in cpp</t>
+  </si>
+  <si>
+    <t>-dangerous of using gets()
+- char src[] = ""Sample Test"";
+char dst[10];
+strcpy(dst, src)</t>
+  </si>
+  <si>
+    <t>File anh Thư</t>
+  </si>
+  <si>
+    <t>What is a template in C++? 
+- class template khác class thường ntn khi compile</t>
+  </si>
+  <si>
+    <t>How do vectors differ from arrays in C++?</t>
+  </si>
+  <si>
+    <t>Unordered_map, map, set, priority_queue, list, …</t>
+  </si>
+  <si>
+    <t>How to loop through map, vector</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Casting in cpp
+- static_cast
+- dynamic_cast
+- reinterpret_cast</t>
+  </si>
+  <si>
+    <t>#27</t>
+  </si>
+  <si>
+    <t>#28</t>
+  </si>
+  <si>
+    <t>#29</t>
+  </si>
+  <si>
+    <t>#30</t>
+  </si>
+  <si>
+    <t>#31</t>
   </si>
 </sst>
 </file>
@@ -4027,7 +4295,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -4176,6 +4444,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4184,6 +4456,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -8621,17 +8899,17 @@
   <sheetData>
     <row r="2" spans="2:17">
       <c r="B2" s="57" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="2:17">
       <c r="C3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" spans="2:17">
       <c r="C4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5" spans="2:17">
@@ -8639,12 +8917,12 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" spans="2:17">
       <c r="D6" s="58" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E6" s="59"/>
       <c r="F6" s="59"/>
@@ -8654,7 +8932,7 @@
       <c r="J6" s="59"/>
       <c r="K6" s="60"/>
       <c r="L6" s="61" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M6" s="44"/>
       <c r="N6" s="44"/>
@@ -8665,7 +8943,7 @@
     <row r="7" spans="2:17">
       <c r="D7" s="59"/>
       <c r="E7" s="59" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F7" s="59"/>
       <c r="G7" s="59"/>
@@ -8675,7 +8953,7 @@
       <c r="K7" s="60"/>
       <c r="L7" s="44"/>
       <c r="M7" s="44" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="N7" s="44"/>
       <c r="O7" s="44"/>
@@ -8685,7 +8963,7 @@
     <row r="8" spans="2:17">
       <c r="D8" s="59"/>
       <c r="E8" s="59" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F8" s="59"/>
       <c r="G8" s="59"/>
@@ -8695,7 +8973,7 @@
       <c r="K8" s="60"/>
       <c r="L8" s="44"/>
       <c r="M8" s="44" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N8" s="44"/>
       <c r="O8" s="44"/>
@@ -8741,7 +9019,7 @@
     <row r="11" spans="2:17">
       <c r="D11" s="59"/>
       <c r="E11" s="59" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F11" s="59"/>
       <c r="G11" s="59"/>
@@ -8751,7 +9029,7 @@
       <c r="K11" s="60"/>
       <c r="L11" s="44"/>
       <c r="M11" s="44" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N11" s="44"/>
       <c r="O11" s="44"/>
@@ -8761,7 +9039,7 @@
     <row r="12" spans="2:17">
       <c r="D12" s="59"/>
       <c r="E12" s="59" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F12" s="59"/>
       <c r="G12" s="59"/>
@@ -8771,7 +9049,7 @@
       <c r="K12" s="60"/>
       <c r="L12" s="44"/>
       <c r="M12" s="44" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="N12" s="44"/>
       <c r="O12" s="44"/>
@@ -8781,7 +9059,7 @@
     <row r="13" spans="2:17">
       <c r="D13" s="59"/>
       <c r="E13" s="59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F13" s="59"/>
       <c r="G13" s="59"/>
@@ -8791,7 +9069,7 @@
       <c r="K13" s="60"/>
       <c r="L13" s="44"/>
       <c r="M13" s="44" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="N13" s="44"/>
       <c r="O13" s="44"/>
@@ -8801,7 +9079,7 @@
     <row r="14" spans="2:17">
       <c r="D14" s="59"/>
       <c r="E14" s="59" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F14" s="59"/>
       <c r="G14" s="59"/>
@@ -8811,7 +9089,7 @@
       <c r="K14" s="60"/>
       <c r="L14" s="44"/>
       <c r="M14" s="44" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="N14" s="44"/>
       <c r="O14" s="44"/>
@@ -8831,7 +9109,7 @@
       <c r="K15" s="60"/>
       <c r="L15" s="44"/>
       <c r="M15" s="44" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N15" s="44"/>
       <c r="O15" s="44"/>
@@ -8861,12 +9139,12 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="19" spans="3:8">
       <c r="E19" s="62" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F19" s="62"/>
       <c r="G19" s="62"/>
@@ -8874,7 +9152,7 @@
     </row>
     <row r="20" spans="3:8">
       <c r="E20" s="62" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F20" s="62"/>
       <c r="G20" s="62"/>
@@ -8882,7 +9160,7 @@
     </row>
     <row r="21" spans="3:8">
       <c r="E21" s="62" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F21" s="62"/>
       <c r="G21" s="62"/>
@@ -8906,28 +9184,28 @@
     </row>
     <row r="25" spans="3:8">
       <c r="D25" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="26" spans="3:8">
       <c r="D26" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="27" spans="3:8">
       <c r="E27" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F27" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="28" spans="3:8">
       <c r="E28" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F28" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="30" spans="3:8">
@@ -8935,7 +9213,7 @@
         <v>3</v>
       </c>
       <c r="D30" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -8956,26 +9234,26 @@
   <sheetData>
     <row r="1" spans="1:5" ht="28.5">
       <c r="A1" s="68" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="23.25">
       <c r="B2" s="63" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="B4" s="71" t="s">
+        <v>336</v>
+      </c>
+      <c r="C4" s="71" t="s">
         <v>337</v>
       </c>
-      <c r="C4" s="71" t="s">
+      <c r="D4" s="71" t="s">
         <v>338</v>
       </c>
-      <c r="D4" s="71" t="s">
-        <v>339</v>
-      </c>
       <c r="E4" s="72" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="45">
@@ -8983,13 +9261,13 @@
         <v>1</v>
       </c>
       <c r="C5" s="70" t="s">
+        <v>339</v>
+      </c>
+      <c r="D5" s="69" t="s">
         <v>340</v>
       </c>
-      <c r="D5" s="69" t="s">
-        <v>341</v>
-      </c>
       <c r="E5" s="69" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="81" customHeight="1">
@@ -8997,13 +9275,13 @@
         <v>2</v>
       </c>
       <c r="C6" s="70" t="s">
+        <v>341</v>
+      </c>
+      <c r="D6" s="69" t="s">
         <v>342</v>
       </c>
-      <c r="D6" s="69" t="s">
-        <v>343</v>
-      </c>
       <c r="E6" s="69" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30">
@@ -9011,32 +9289,32 @@
         <v>3</v>
       </c>
       <c r="C7" s="70" t="s">
+        <v>343</v>
+      </c>
+      <c r="D7" s="69" t="s">
         <v>344</v>
       </c>
-      <c r="D7" s="69" t="s">
-        <v>345</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="23.25">
       <c r="B10" s="63" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="B12" s="73" t="s">
+        <v>336</v>
+      </c>
+      <c r="C12" s="73" t="s">
         <v>337</v>
       </c>
-      <c r="C12" s="73" t="s">
+      <c r="D12" s="73" t="s">
         <v>338</v>
       </c>
-      <c r="D12" s="73" t="s">
-        <v>339</v>
-      </c>
       <c r="E12" s="74" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30">
@@ -9044,13 +9322,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="70" t="s">
+        <v>346</v>
+      </c>
+      <c r="D13" s="69" t="s">
         <v>347</v>
       </c>
-      <c r="D13" s="69" t="s">
-        <v>348</v>
-      </c>
       <c r="E13" s="69" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30">
@@ -9058,13 +9336,13 @@
         <v>2</v>
       </c>
       <c r="C14" s="70" t="s">
+        <v>348</v>
+      </c>
+      <c r="D14" s="69" t="s">
         <v>349</v>
       </c>
-      <c r="D14" s="69" t="s">
-        <v>350</v>
-      </c>
       <c r="E14" s="69" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30">
@@ -9072,13 +9350,13 @@
         <v>3</v>
       </c>
       <c r="C15" s="70" t="s">
+        <v>350</v>
+      </c>
+      <c r="D15" s="69" t="s">
         <v>351</v>
       </c>
-      <c r="D15" s="69" t="s">
-        <v>352</v>
-      </c>
       <c r="E15" s="69" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30">
@@ -9086,13 +9364,13 @@
         <v>4</v>
       </c>
       <c r="C16" s="70" t="s">
+        <v>352</v>
+      </c>
+      <c r="D16" s="69" t="s">
         <v>353</v>
       </c>
-      <c r="D16" s="69" t="s">
-        <v>354</v>
-      </c>
       <c r="E16" s="75" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="165">
@@ -9100,13 +9378,13 @@
         <v>5</v>
       </c>
       <c r="C17" s="70" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D17" s="69" t="s">
+        <v>430</v>
+      </c>
+      <c r="E17" s="75" t="s">
         <v>431</v>
-      </c>
-      <c r="E17" s="75" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="180">
@@ -9114,13 +9392,13 @@
         <v>6</v>
       </c>
       <c r="C18" s="70" t="s">
+        <v>355</v>
+      </c>
+      <c r="D18" s="69" t="s">
         <v>356</v>
       </c>
-      <c r="D18" s="69" t="s">
-        <v>357</v>
-      </c>
       <c r="E18" s="75" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="135">
@@ -9128,13 +9406,13 @@
         <v>7</v>
       </c>
       <c r="C19" s="70" t="s">
+        <v>357</v>
+      </c>
+      <c r="D19" s="69" t="s">
         <v>358</v>
       </c>
-      <c r="D19" s="69" t="s">
-        <v>359</v>
-      </c>
       <c r="E19" s="75" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="135">
@@ -9142,32 +9420,32 @@
         <v>8</v>
       </c>
       <c r="C20" s="70" t="s">
+        <v>359</v>
+      </c>
+      <c r="D20" s="69" t="s">
         <v>360</v>
       </c>
-      <c r="D20" s="69" t="s">
-        <v>361</v>
-      </c>
       <c r="E20" s="75" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="23.25">
       <c r="B23" s="63" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" s="73" t="s">
+        <v>336</v>
+      </c>
+      <c r="C25" s="73" t="s">
         <v>337</v>
       </c>
-      <c r="C25" s="73" t="s">
+      <c r="D25" s="73" t="s">
         <v>338</v>
       </c>
-      <c r="D25" s="73" t="s">
-        <v>339</v>
-      </c>
       <c r="E25" s="74" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="26" spans="2:5">
@@ -9175,10 +9453,10 @@
         <v>1</v>
       </c>
       <c r="C26" s="70" t="s">
+        <v>361</v>
+      </c>
+      <c r="D26" s="69" t="s">
         <v>362</v>
-      </c>
-      <c r="D26" s="69" t="s">
-        <v>363</v>
       </c>
       <c r="E26" s="1"/>
     </row>
@@ -9187,10 +9465,10 @@
         <v>2</v>
       </c>
       <c r="C27" s="70" t="s">
+        <v>363</v>
+      </c>
+      <c r="D27" s="69" t="s">
         <v>364</v>
-      </c>
-      <c r="D27" s="69" t="s">
-        <v>365</v>
       </c>
       <c r="E27" s="1"/>
     </row>
@@ -9199,10 +9477,10 @@
         <v>3</v>
       </c>
       <c r="C28" s="70" t="s">
+        <v>365</v>
+      </c>
+      <c r="D28" s="69" t="s">
         <v>366</v>
-      </c>
-      <c r="D28" s="69" t="s">
-        <v>367</v>
       </c>
       <c r="E28" s="1"/>
     </row>
@@ -9211,27 +9489,27 @@
         <v>4</v>
       </c>
       <c r="C29" s="70" t="s">
+        <v>367</v>
+      </c>
+      <c r="D29" s="69" t="s">
         <v>368</v>
-      </c>
-      <c r="D29" s="69" t="s">
-        <v>369</v>
       </c>
       <c r="E29" s="1"/>
     </row>
     <row r="32" spans="2:5" ht="23.25">
       <c r="B32" s="63" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="34" spans="2:4">
       <c r="B34" s="64" t="s">
+        <v>336</v>
+      </c>
+      <c r="C34" s="64" t="s">
         <v>337</v>
       </c>
-      <c r="C34" s="64" t="s">
+      <c r="D34" s="64" t="s">
         <v>338</v>
-      </c>
-      <c r="D34" s="64" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="30">
@@ -9239,10 +9517,10 @@
         <v>1</v>
       </c>
       <c r="C35" s="66" t="s">
+        <v>369</v>
+      </c>
+      <c r="D35" s="65" t="s">
         <v>370</v>
-      </c>
-      <c r="D35" s="65" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="36" spans="2:4">
@@ -9250,10 +9528,10 @@
         <v>2</v>
       </c>
       <c r="C36" s="66" t="s">
+        <v>371</v>
+      </c>
+      <c r="D36" s="65" t="s">
         <v>372</v>
-      </c>
-      <c r="D36" s="65" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="37" spans="2:4" ht="30">
@@ -9261,10 +9539,10 @@
         <v>3</v>
       </c>
       <c r="C37" s="66" t="s">
+        <v>373</v>
+      </c>
+      <c r="D37" s="65" t="s">
         <v>374</v>
-      </c>
-      <c r="D37" s="65" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="38" spans="2:4">
@@ -9272,26 +9550,26 @@
         <v>4</v>
       </c>
       <c r="C38" s="66" t="s">
+        <v>375</v>
+      </c>
+      <c r="D38" s="65" t="s">
         <v>376</v>
-      </c>
-      <c r="D38" s="65" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="41" spans="2:4" ht="23.25">
       <c r="B41" s="63" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="43" spans="2:4">
       <c r="B43" s="64" t="s">
+        <v>336</v>
+      </c>
+      <c r="C43" s="64" t="s">
         <v>337</v>
       </c>
-      <c r="C43" s="64" t="s">
+      <c r="D43" s="64" t="s">
         <v>338</v>
-      </c>
-      <c r="D43" s="64" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="44" spans="2:4" ht="30">
@@ -9299,10 +9577,10 @@
         <v>1</v>
       </c>
       <c r="C44" s="66" t="s">
+        <v>377</v>
+      </c>
+      <c r="D44" s="65" t="s">
         <v>378</v>
-      </c>
-      <c r="D44" s="65" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="45" spans="2:4">
@@ -9310,10 +9588,10 @@
         <v>2</v>
       </c>
       <c r="C45" s="66" t="s">
+        <v>379</v>
+      </c>
+      <c r="D45" s="65" t="s">
         <v>380</v>
-      </c>
-      <c r="D45" s="65" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="46" spans="2:4">
@@ -9321,10 +9599,10 @@
         <v>3</v>
       </c>
       <c r="C46" s="67" t="s">
+        <v>381</v>
+      </c>
+      <c r="D46" s="65" t="s">
         <v>382</v>
-      </c>
-      <c r="D46" s="65" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="47" spans="2:4">
@@ -9332,26 +9610,26 @@
         <v>4</v>
       </c>
       <c r="C47" s="67" t="s">
+        <v>383</v>
+      </c>
+      <c r="D47" s="65" t="s">
         <v>384</v>
-      </c>
-      <c r="D47" s="65" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="50" spans="2:4" ht="23.25">
       <c r="B50" s="63" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="52" spans="2:4">
       <c r="B52" s="64" t="s">
+        <v>336</v>
+      </c>
+      <c r="C52" s="64" t="s">
         <v>337</v>
       </c>
-      <c r="C52" s="64" t="s">
+      <c r="D52" s="64" t="s">
         <v>338</v>
-      </c>
-      <c r="D52" s="64" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="53" spans="2:4">
@@ -9359,10 +9637,10 @@
         <v>1</v>
       </c>
       <c r="C53" s="66" t="s">
+        <v>385</v>
+      </c>
+      <c r="D53" s="65" t="s">
         <v>386</v>
-      </c>
-      <c r="D53" s="65" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="54" spans="2:4">
@@ -9370,10 +9648,10 @@
         <v>2</v>
       </c>
       <c r="C54" s="66" t="s">
+        <v>387</v>
+      </c>
+      <c r="D54" s="65" t="s">
         <v>388</v>
-      </c>
-      <c r="D54" s="65" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="55" spans="2:4">
@@ -9381,10 +9659,10 @@
         <v>3</v>
       </c>
       <c r="C55" s="66" t="s">
+        <v>389</v>
+      </c>
+      <c r="D55" s="65" t="s">
         <v>390</v>
-      </c>
-      <c r="D55" s="65" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="56" spans="2:4">
@@ -9392,18 +9670,18 @@
     </row>
     <row r="58" spans="2:4" ht="23.25">
       <c r="B58" s="63" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="60" spans="2:4">
       <c r="B60" s="64" t="s">
+        <v>336</v>
+      </c>
+      <c r="C60" s="64" t="s">
         <v>337</v>
       </c>
-      <c r="C60" s="64" t="s">
+      <c r="D60" s="64" t="s">
         <v>338</v>
-      </c>
-      <c r="D60" s="64" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="61" spans="2:4">
@@ -9411,10 +9689,10 @@
         <v>1</v>
       </c>
       <c r="C61" s="66" t="s">
+        <v>391</v>
+      </c>
+      <c r="D61" s="65" t="s">
         <v>392</v>
-      </c>
-      <c r="D61" s="65" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="62" spans="2:4" ht="45">
@@ -9422,10 +9700,10 @@
         <v>2</v>
       </c>
       <c r="C62" s="66" t="s">
+        <v>393</v>
+      </c>
+      <c r="D62" s="65" t="s">
         <v>394</v>
-      </c>
-      <c r="D62" s="65" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="63" spans="2:4" ht="30">
@@ -9433,10 +9711,10 @@
         <v>3</v>
       </c>
       <c r="C63" s="66" t="s">
+        <v>395</v>
+      </c>
+      <c r="D63" s="65" t="s">
         <v>396</v>
-      </c>
-      <c r="D63" s="65" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="64" spans="2:4">
@@ -9444,10 +9722,10 @@
         <v>4</v>
       </c>
       <c r="C64" s="66" t="s">
+        <v>397</v>
+      </c>
+      <c r="D64" s="65" t="s">
         <v>398</v>
-      </c>
-      <c r="D64" s="65" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="65" spans="2:4">
@@ -9455,26 +9733,26 @@
         <v>5</v>
       </c>
       <c r="C65" s="66" t="s">
+        <v>399</v>
+      </c>
+      <c r="D65" s="65" t="s">
         <v>400</v>
-      </c>
-      <c r="D65" s="65" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="68" spans="2:4" ht="23.25">
       <c r="B68" s="63" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="70" spans="2:4">
       <c r="B70" s="64" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C70" s="64" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D70" s="64" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="71" spans="2:4">
@@ -9482,10 +9760,10 @@
         <v>1</v>
       </c>
       <c r="C71" s="65" t="s">
+        <v>403</v>
+      </c>
+      <c r="D71" s="65" t="s">
         <v>404</v>
-      </c>
-      <c r="D71" s="65" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="72" spans="2:4">
@@ -9493,10 +9771,10 @@
         <v>2</v>
       </c>
       <c r="C72" s="65" t="s">
+        <v>405</v>
+      </c>
+      <c r="D72" s="65" t="s">
         <v>406</v>
-      </c>
-      <c r="D72" s="65" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="73" spans="2:4">
@@ -9504,10 +9782,10 @@
         <v>3</v>
       </c>
       <c r="C73" s="65" t="s">
+        <v>407</v>
+      </c>
+      <c r="D73" s="65" t="s">
         <v>408</v>
-      </c>
-      <c r="D73" s="65" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="74" spans="2:4">
@@ -9515,10 +9793,10 @@
         <v>4</v>
       </c>
       <c r="C74" s="65" t="s">
+        <v>409</v>
+      </c>
+      <c r="D74" s="65" t="s">
         <v>410</v>
-      </c>
-      <c r="D74" s="65" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="75" spans="2:4">
@@ -9526,10 +9804,10 @@
         <v>5</v>
       </c>
       <c r="C75" s="65" t="s">
+        <v>411</v>
+      </c>
+      <c r="D75" s="65" t="s">
         <v>412</v>
-      </c>
-      <c r="D75" s="65" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="76" spans="2:4">
@@ -9537,10 +9815,57 @@
         <v>6</v>
       </c>
       <c r="C76" s="65" t="s">
+        <v>413</v>
+      </c>
+      <c r="D76" s="65" t="s">
         <v>414</v>
       </c>
-      <c r="D76" s="65" t="s">
-        <v>415</v>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="B2" s="6" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4">
+      <c r="C3" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4">
+      <c r="C4" s="76" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="B5" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="C6" t="s">
+        <v>446</v>
+      </c>
+      <c r="D6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="C7" t="s">
+        <v>447</v>
+      </c>
+      <c r="D7" t="s">
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -10702,7 +11027,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:G54"/>
+  <dimension ref="B1:G90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="50.140625" bestFit="1" customWidth="1"/>
@@ -11050,7 +11375,9 @@
       <c r="C23" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="D23" s="6"/>
+      <c r="D23" s="42">
+        <v>1</v>
+      </c>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
     </row>
@@ -11405,7 +11732,7 @@
         <v>266</v>
       </c>
       <c r="C47" s="57" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D47" s="42">
         <v>1</v>
@@ -11417,13 +11744,13 @@
     </row>
     <row r="48" spans="2:6">
       <c r="B48" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C48" s="56" t="s">
-        <v>302</v>
-      </c>
-      <c r="D48" s="42">
-        <v>0</v>
+        <v>301</v>
+      </c>
+      <c r="D48" s="51">
+        <v>0.8</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="16" t="s">
@@ -11432,10 +11759,10 @@
     </row>
     <row r="49" spans="2:6">
       <c r="B49" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
@@ -11443,7 +11770,7 @@
     </row>
     <row r="50" spans="2:6">
       <c r="B50" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>286</v>
@@ -11452,32 +11779,36 @@
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
     </row>
-    <row r="51" spans="2:6">
+    <row r="51" spans="2:6" ht="30">
       <c r="B51" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>287</v>
+        <v>321</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>437</v>
       </c>
       <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
+      <c r="E51" s="16" t="s">
+        <v>438</v>
+      </c>
       <c r="F51" s="6"/>
     </row>
     <row r="52" spans="2:6">
       <c r="B52" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>290</v>
+        <v>439</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
     </row>
     <row r="53" spans="2:6">
-      <c r="B53" s="5"/>
+      <c r="B53" s="5" t="s">
+        <v>323</v>
+      </c>
       <c r="C53" s="6" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
@@ -11485,14 +11816,426 @@
     </row>
     <row r="54" spans="2:6">
       <c r="B54" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="D54" s="42">
+        <v>1</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6">
+      <c r="B55" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+    </row>
+    <row r="56" spans="2:6">
+      <c r="B56" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="D56" s="6"/>
+      <c r="E56" s="16" t="s">
+        <v>471</v>
+      </c>
+      <c r="F56" s="6"/>
+    </row>
+    <row r="57" spans="2:6">
+      <c r="B57" s="5">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="D57" s="6"/>
+      <c r="E57" s="16"/>
+      <c r="F57" s="6"/>
+    </row>
+    <row r="58" spans="2:6">
+      <c r="B58" s="5">
+        <v>16.2</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+    </row>
+    <row r="59" spans="2:6">
+      <c r="B59" s="5">
+        <v>16.3</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6"/>
+      <c r="F59" s="6"/>
+    </row>
+    <row r="60" spans="2:6">
+      <c r="B60" s="5">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+    </row>
+    <row r="61" spans="2:6">
+      <c r="B61" s="5">
+        <v>16.5</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+    </row>
+    <row r="62" spans="2:6">
+      <c r="B62" s="5">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="D62" s="6"/>
+      <c r="E62" s="6"/>
+      <c r="F62" s="6"/>
+    </row>
+    <row r="63" spans="2:6" ht="40.5" customHeight="1">
+      <c r="B63" s="5">
+        <v>16.7</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
+    </row>
+    <row r="64" spans="2:6">
+      <c r="B64" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+    </row>
+    <row r="65" spans="2:6" ht="30">
+      <c r="B65" s="5">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="C65" s="81" t="s">
+        <v>490</v>
+      </c>
+      <c r="D65" s="6"/>
+      <c r="E65" s="6"/>
+      <c r="F65" s="6"/>
+    </row>
+    <row r="66" spans="2:6" ht="30">
+      <c r="B66" s="5">
+        <v>17.2</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
+    </row>
+    <row r="67" spans="2:6" ht="50.25" customHeight="1">
+      <c r="B67" s="5">
+        <v>17.3</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="D67" s="6"/>
+      <c r="E67" s="16" t="s">
+        <v>471</v>
+      </c>
+      <c r="F67" s="6"/>
+    </row>
+    <row r="68" spans="2:6" ht="30">
+      <c r="B68" s="5">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>461</v>
+      </c>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
+    </row>
+    <row r="69" spans="2:6">
+      <c r="B69" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="6"/>
+    </row>
+    <row r="70" spans="2:6">
+      <c r="B70" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+    </row>
+    <row r="71" spans="2:6">
+      <c r="B71" s="5">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="D71" s="6"/>
+      <c r="E71" s="6"/>
+      <c r="F71" s="6"/>
+    </row>
+    <row r="72" spans="2:6">
+      <c r="B72" s="5">
+        <v>18.2</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="D72" s="6"/>
+      <c r="E72" s="6"/>
+      <c r="F72" s="6"/>
+    </row>
+    <row r="73" spans="2:6">
+      <c r="B73" s="5">
+        <v>18.3</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="D73" s="6"/>
+      <c r="E73" s="6"/>
+      <c r="F73" s="6"/>
+    </row>
+    <row r="74" spans="2:6">
+      <c r="B74" s="5">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="D74" s="6"/>
+      <c r="E74" s="6"/>
+      <c r="F74" s="6"/>
+    </row>
+    <row r="75" spans="2:6">
+      <c r="B75" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="D75" s="6"/>
+      <c r="E75" s="6"/>
+      <c r="F75" s="6"/>
+    </row>
+    <row r="76" spans="2:6">
+      <c r="B76" s="5">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="D76" s="6"/>
+      <c r="E76" s="6"/>
+      <c r="F76" s="6"/>
+    </row>
+    <row r="77" spans="2:6">
+      <c r="B77" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="D77" s="6"/>
+      <c r="E77" s="6"/>
+      <c r="F77" s="6"/>
+    </row>
+    <row r="78" spans="2:6">
+      <c r="B78" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="D78" s="6"/>
+      <c r="E78" s="6"/>
+      <c r="F78" s="6"/>
+    </row>
+    <row r="79" spans="2:6">
+      <c r="B79" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="D79" s="6"/>
+      <c r="E79" s="6"/>
+      <c r="F79" s="6"/>
+    </row>
+    <row r="80" spans="2:6" ht="30">
+      <c r="B80" s="5">
+        <v>21.2</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="D80" s="6"/>
+      <c r="E80" s="6"/>
+      <c r="F80" s="6"/>
+    </row>
+    <row r="81" spans="2:6">
+      <c r="B81" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="C81" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="C54" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
+      <c r="D81" s="6"/>
+      <c r="E81" s="16" t="s">
+        <v>475</v>
+      </c>
+      <c r="F81" s="6"/>
+    </row>
+    <row r="82" spans="2:6">
+      <c r="B82" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="D82" s="6"/>
+      <c r="E82" s="16" t="s">
+        <v>475</v>
+      </c>
+      <c r="F82" s="6"/>
+    </row>
+    <row r="83" spans="2:6">
+      <c r="B83" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="D83" s="6"/>
+      <c r="E83" s="16"/>
+      <c r="F83" s="6"/>
+    </row>
+    <row r="84" spans="2:6">
+      <c r="B84" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="D84" s="6"/>
+      <c r="E84" s="16"/>
+      <c r="F84" s="6"/>
+    </row>
+    <row r="85" spans="2:6" ht="60">
+      <c r="B85" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="C85" s="82" t="s">
+        <v>491</v>
+      </c>
+      <c r="D85" s="6"/>
+      <c r="E85" s="16" t="s">
+        <v>492</v>
+      </c>
+      <c r="F85" s="6"/>
+    </row>
+    <row r="86" spans="2:6" ht="30">
+      <c r="B86" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="D86" s="6"/>
+      <c r="E86" s="16"/>
+      <c r="F86" s="6"/>
+    </row>
+    <row r="87" spans="2:6">
+      <c r="B87" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="D87" s="6"/>
+      <c r="E87" s="16"/>
+      <c r="F87" s="6"/>
+    </row>
+    <row r="88" spans="2:6" ht="60">
+      <c r="B88" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>497</v>
+      </c>
+      <c r="D88" s="6"/>
+      <c r="E88" s="16"/>
+      <c r="F88" s="6"/>
+    </row>
+    <row r="89" spans="2:6" ht="30">
+      <c r="B89" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="D89" s="6"/>
+      <c r="E89" s="16"/>
+      <c r="F89" s="6"/>
+    </row>
+    <row r="90" spans="2:6">
+      <c r="B90" s="77" t="s">
+        <v>482</v>
+      </c>
+      <c r="C90" s="57" t="s">
+        <v>481</v>
+      </c>
+      <c r="D90" s="1"/>
+      <c r="E90" s="49" t="s">
+        <v>480</v>
+      </c>
+      <c r="F90" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11540,9 +12283,16 @@
     <hyperlink ref="F46" location="'#6'!B33" display="Link"/>
     <hyperlink ref="F47" location="'#7'!B2" display="Link"/>
     <hyperlink ref="F48" location="'#8'!A1" display="Link"/>
+    <hyperlink ref="E51" r:id="rId6"/>
+    <hyperlink ref="F54" location="'#14'!B2" display="Link"/>
+    <hyperlink ref="E56" r:id="rId7"/>
+    <hyperlink ref="E67" r:id="rId8"/>
+    <hyperlink ref="E81" r:id="rId9"/>
+    <hyperlink ref="E82" r:id="rId10"/>
+    <hyperlink ref="E90" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId12"/>
 </worksheet>
 </file>
 
@@ -11857,7 +12607,7 @@
       <c r="D12" s="11"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1">
-      <c r="C13" s="76" t="s">
+      <c r="C13" s="78" t="s">
         <v>78</v>
       </c>
       <c r="D13" s="26" t="s">
@@ -11874,7 +12624,7 @@
       <c r="I13" s="25"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" thickBot="1">
-      <c r="C14" s="77"/>
+      <c r="C14" s="79"/>
       <c r="D14" s="23" t="s">
         <v>65</v>
       </c>
@@ -11890,7 +12640,7 @@
       <c r="J14" s="25"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="C15" s="77"/>
+      <c r="C15" s="79"/>
       <c r="D15" s="26" t="s">
         <v>66</v>
       </c>
@@ -11905,7 +12655,7 @@
       <c r="I15" s="28"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="C16" s="77"/>
+      <c r="C16" s="79"/>
       <c r="D16" s="29"/>
       <c r="E16" s="30" t="s">
         <v>74</v>
@@ -11916,7 +12666,7 @@
       <c r="I16" s="31"/>
     </row>
     <row r="17" spans="3:12" ht="15.75" thickBot="1">
-      <c r="C17" s="78"/>
+      <c r="C17" s="80"/>
       <c r="D17" s="32"/>
       <c r="E17" s="33" t="s">
         <v>75</v>
@@ -11947,7 +12697,7 @@
       <c r="L18" s="25"/>
     </row>
     <row r="19" spans="3:12" ht="15.75" thickBot="1">
-      <c r="C19" s="76" t="s">
+      <c r="C19" s="78" t="s">
         <v>78</v>
       </c>
       <c r="D19" s="23" t="s">
@@ -11958,7 +12708,7 @@
       </c>
     </row>
     <row r="20" spans="3:12">
-      <c r="C20" s="77"/>
+      <c r="C20" s="79"/>
       <c r="D20" s="26" t="s">
         <v>82</v>
       </c>
@@ -11967,7 +12717,7 @@
       </c>
     </row>
     <row r="21" spans="3:12" ht="15.75" thickBot="1">
-      <c r="C21" s="78"/>
+      <c r="C21" s="80"/>
       <c r="D21" s="32"/>
       <c r="E21" s="40" t="s">
         <v>84</v>
@@ -13118,7 +13868,7 @@
         <v>272</v>
       </c>
       <c r="E5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" spans="2:26">
@@ -13146,7 +13896,7 @@
         <v>277</v>
       </c>
       <c r="F12" s="55" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G12" s="55"/>
       <c r="H12" s="55"/>
@@ -13211,39 +13961,39 @@
     </row>
     <row r="35" spans="2:7">
       <c r="C35" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="37" spans="2:7">
       <c r="D37" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E37" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="38" spans="2:7">
       <c r="D38" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E38" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="39" spans="2:7">
       <c r="D39" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E39" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="40" spans="2:7">
       <c r="D40" t="s">
+        <v>299</v>
+      </c>
+      <c r="G40" t="s">
         <v>300</v>
-      </c>
-      <c r="G40" t="s">
-        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
anhdxh fix tren xe
</commit_message>
<xml_diff>
--- a/Study_CL.xlsx
+++ b/Study_CL.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="16"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Knowhow" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="610">
   <si>
     <t>No.</t>
   </si>
@@ -5143,6 +5143,95 @@
   </si>
   <si>
     <t>gcovr -r .. --html --html-details -o coverage.html</t>
+  </si>
+  <si>
+    <t>Tùy vào đối số truyền vào hàm mà chương trình sẽ ngầm hiểu là hàm đang được dùng theo cách nào</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Overloading</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Nạp chồng hàm, là cơ chế trong C++ cho phép nhiều cách xử lý khác nhau cho cùng 1 tên hàm. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Overriding </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Ghi đè hàm, là cơ chế trong C++ mà khi kết hợp với phương thức virtual cho phép hàm cùng tên</t>
+    </r>
+  </si>
+  <si>
+    <t>trong class con, mặc dù có cùng tham số, đối số truyền vào, kiểu trả về nhưng có xử lý khác so với hàm cùng tên trong class cha</t>
+  </si>
+  <si>
+    <t>Khâu hoạt động</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Thời điểm quyết định : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Compile-time</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Thời điểm quyết định : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Runtime</t>
+    </r>
+  </si>
+  <si>
+    <t>Mục đích : Tăng tính linh hoạt cho code</t>
+  </si>
+  <si>
+    <t>Mục đích : Thay đổi hành vi của class cha</t>
   </si>
 </sst>
 </file>
@@ -9914,19 +10003,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:K22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="5.7109375" customWidth="1"/>
-    <col min="3" max="3" width="37.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.42578125" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" customWidth="1"/>
+    <col min="3" max="3" width="37.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.453125" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="18.75">
+    <row r="2" spans="2:11" ht="18.5">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -9952,7 +10041,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="2:11" ht="45">
+    <row r="3" spans="2:11" ht="43.5">
       <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
@@ -10306,9 +10395,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:Q30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="11" max="11" width="3.7109375" customWidth="1"/>
+    <col min="11" max="11" width="3.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:17">
@@ -10638,12 +10727,12 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E76"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="4.42578125" customWidth="1"/>
-    <col min="3" max="3" width="39.7109375" customWidth="1"/>
-    <col min="4" max="4" width="50.85546875" customWidth="1"/>
-    <col min="5" max="5" width="75.42578125" customWidth="1"/>
+    <col min="2" max="2" width="4.453125" customWidth="1"/>
+    <col min="3" max="3" width="39.7265625" customWidth="1"/>
+    <col min="4" max="4" width="50.81640625" customWidth="1"/>
+    <col min="5" max="5" width="75.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.5">
@@ -10651,7 +10740,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="23.25">
+    <row r="2" spans="1:5" ht="23.5">
       <c r="B2" s="63" t="s">
         <v>420</v>
       </c>
@@ -10670,7 +10759,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="45">
+    <row r="5" spans="1:5" ht="43.5">
       <c r="B5" s="69">
         <v>1</v>
       </c>
@@ -10698,7 +10787,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30">
+    <row r="7" spans="1:5" ht="29">
       <c r="B7" s="69">
         <v>3</v>
       </c>
@@ -10712,7 +10801,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="23.25">
+    <row r="10" spans="1:5" ht="23.5">
       <c r="B10" s="63" t="s">
         <v>344</v>
       </c>
@@ -10731,7 +10820,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="30">
+    <row r="13" spans="1:5">
       <c r="B13" s="69">
         <v>1</v>
       </c>
@@ -10745,7 +10834,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="30">
+    <row r="14" spans="1:5" ht="29">
       <c r="B14" s="69">
         <v>2</v>
       </c>
@@ -10759,7 +10848,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30">
+    <row r="15" spans="1:5" ht="29">
       <c r="B15" s="69">
         <v>3</v>
       </c>
@@ -10773,7 +10862,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30">
+    <row r="16" spans="1:5" ht="29">
       <c r="B16" s="69">
         <v>4</v>
       </c>
@@ -10787,7 +10876,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="165">
+    <row r="17" spans="2:5" ht="145">
       <c r="B17" s="69">
         <v>5</v>
       </c>
@@ -10801,7 +10890,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="180">
+    <row r="18" spans="2:5" ht="159.5">
       <c r="B18" s="69">
         <v>6</v>
       </c>
@@ -10815,7 +10904,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="135">
+    <row r="19" spans="2:5" ht="130.5">
       <c r="B19" s="69">
         <v>7</v>
       </c>
@@ -10829,7 +10918,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="135">
+    <row r="20" spans="2:5" ht="130.5">
       <c r="B20" s="69">
         <v>8</v>
       </c>
@@ -10843,7 +10932,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="23.25">
+    <row r="23" spans="2:5" ht="23.5">
       <c r="B23" s="63" t="s">
         <v>419</v>
       </c>
@@ -10910,7 +10999,7 @@
       </c>
       <c r="E29" s="1"/>
     </row>
-    <row r="32" spans="2:5" ht="23.25">
+    <row r="32" spans="2:5" ht="23.5">
       <c r="B32" s="63" t="s">
         <v>418</v>
       </c>
@@ -10926,7 +11015,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="35" spans="2:4" ht="30">
+    <row r="35" spans="2:4" ht="29">
       <c r="B35" s="65">
         <v>1</v>
       </c>
@@ -10948,7 +11037,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="37" spans="2:4" ht="30">
+    <row r="37" spans="2:4">
       <c r="B37" s="65">
         <v>3</v>
       </c>
@@ -10970,7 +11059,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="41" spans="2:4" ht="23.25">
+    <row r="41" spans="2:4" ht="23.5">
       <c r="B41" s="63" t="s">
         <v>417</v>
       </c>
@@ -10986,7 +11075,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="44" spans="2:4" ht="30">
+    <row r="44" spans="2:4">
       <c r="B44" s="65">
         <v>1</v>
       </c>
@@ -11030,7 +11119,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="50" spans="2:4" ht="23.25">
+    <row r="50" spans="2:4" ht="23.5">
       <c r="B50" s="63" t="s">
         <v>416</v>
       </c>
@@ -11082,7 +11171,7 @@
     <row r="56" spans="2:4">
       <c r="B56" s="65"/>
     </row>
-    <row r="58" spans="2:4" ht="23.25">
+    <row r="58" spans="2:4" ht="23.5">
       <c r="B58" s="63" t="s">
         <v>415</v>
       </c>
@@ -11109,7 +11198,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="62" spans="2:4" ht="45">
+    <row r="62" spans="2:4" ht="29">
       <c r="B62" s="65">
         <v>2</v>
       </c>
@@ -11120,7 +11209,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="63" spans="2:4" ht="30">
+    <row r="63" spans="2:4" ht="29">
       <c r="B63" s="65">
         <v>3</v>
       </c>
@@ -11153,7 +11242,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="68" spans="2:4" ht="23.25">
+    <row r="68" spans="2:4" ht="23.5">
       <c r="B68" s="63" t="s">
         <v>400</v>
       </c>
@@ -11244,7 +11333,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:S38"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
@@ -11571,7 +11660,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:M57"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
@@ -11885,7 +11974,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:E25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
@@ -12002,7 +12091,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" s="6" t="s">
@@ -12017,7 +12106,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:D7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:4">
       <c r="B2" s="6" t="s">
@@ -12063,8 +12152,8 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:D10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="B2:D20"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:4">
       <c r="B2" s="6" t="s">
@@ -12100,23 +12189,69 @@
         <v>465</v>
       </c>
     </row>
+    <row r="11" spans="2:4">
+      <c r="C11" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4">
+      <c r="C12" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="C13" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="C14" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="C16" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" t="s">
+        <v>609</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F103"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.26953125" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="5" max="5" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="18.75">
+    <row r="2" spans="2:6" ht="18.5">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -13259,12 +13394,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:G90"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="50.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="68.5703125" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+    <col min="3" max="3" width="50.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="68.54296875" customWidth="1"/>
+    <col min="6" max="6" width="9.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6">
@@ -13272,7 +13407,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="2:6" ht="18.75">
+    <row r="2" spans="2:6" ht="18.5">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -14018,7 +14153,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51" spans="2:6" ht="30">
+    <row r="51" spans="2:6" ht="29">
       <c r="B51" s="5" t="s">
         <v>320</v>
       </c>
@@ -14120,7 +14255,9 @@
       <c r="C58" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="D58" s="6"/>
+      <c r="D58" s="42">
+        <v>1</v>
+      </c>
       <c r="E58" s="6"/>
       <c r="F58" s="16" t="s">
         <v>14</v>
@@ -14192,7 +14329,7 @@
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
     </row>
-    <row r="65" spans="2:6" ht="30">
+    <row r="65" spans="2:6" ht="29">
       <c r="B65" s="5">
         <v>17.100000000000001</v>
       </c>
@@ -14203,7 +14340,7 @@
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
     </row>
-    <row r="66" spans="2:6" ht="30">
+    <row r="66" spans="2:6" ht="29">
       <c r="B66" s="5">
         <v>17.2</v>
       </c>
@@ -14227,7 +14364,7 @@
       </c>
       <c r="F67" s="6"/>
     </row>
-    <row r="68" spans="2:6" ht="30">
+    <row r="68" spans="2:6" ht="29">
       <c r="B68" s="5">
         <v>17.399999999999999</v>
       </c>
@@ -14359,7 +14496,7 @@
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
     </row>
-    <row r="80" spans="2:6" ht="30">
+    <row r="80" spans="2:6" ht="29">
       <c r="B80" s="5">
         <v>21.2</v>
       </c>
@@ -14418,7 +14555,7 @@
       <c r="E84" s="16"/>
       <c r="F84" s="6"/>
     </row>
-    <row r="85" spans="2:6" ht="60">
+    <row r="85" spans="2:6" ht="58">
       <c r="B85" s="5" t="s">
         <v>495</v>
       </c>
@@ -14431,7 +14568,7 @@
       </c>
       <c r="F85" s="6"/>
     </row>
-    <row r="86" spans="2:6" ht="30">
+    <row r="86" spans="2:6" ht="29">
       <c r="B86" s="5" t="s">
         <v>496</v>
       </c>
@@ -14453,7 +14590,7 @@
       <c r="E87" s="16"/>
       <c r="F87" s="6"/>
     </row>
-    <row r="88" spans="2:6" ht="60">
+    <row r="88" spans="2:6" ht="58">
       <c r="B88" s="5" t="s">
         <v>498</v>
       </c>
@@ -14464,7 +14601,7 @@
       <c r="E88" s="16"/>
       <c r="F88" s="6"/>
     </row>
-    <row r="89" spans="2:6" ht="30">
+    <row r="89" spans="2:6" ht="29">
       <c r="B89" s="5" t="s">
         <v>499</v>
       </c>
@@ -14556,13 +14693,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J164"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="4.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" customWidth="1"/>
+    <col min="1" max="1" width="4.26953125" customWidth="1"/>
+    <col min="2" max="2" width="6.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75">
+    <row r="1" spans="1:3" ht="18.5">
       <c r="C1" s="41" t="s">
         <v>15</v>
       </c>
@@ -14819,14 +14956,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="3" max="3" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" customWidth="1"/>
-    <col min="5" max="5" width="48.85546875" customWidth="1"/>
+    <col min="3" max="3" width="10.453125" customWidth="1"/>
+    <col min="4" max="4" width="5.26953125" customWidth="1"/>
+    <col min="5" max="5" width="48.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75">
+    <row r="1" spans="1:10" ht="18.5">
       <c r="C1" s="41" t="s">
         <v>57</v>
       </c>
@@ -14857,13 +14994,13 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.75" thickBot="1">
+    <row r="12" spans="1:10" ht="15" thickBot="1">
       <c r="C12" s="11" t="s">
         <v>63</v>
       </c>
       <c r="D12" s="11"/>
     </row>
-    <row r="13" spans="1:10" ht="15.75" thickBot="1">
+    <row r="13" spans="1:10" ht="15" thickBot="1">
       <c r="C13" s="92" t="s">
         <v>78</v>
       </c>
@@ -14880,7 +15017,7 @@
       <c r="H13" s="24"/>
       <c r="I13" s="25"/>
     </row>
-    <row r="14" spans="1:10" ht="15.75" thickBot="1">
+    <row r="14" spans="1:10" ht="15" thickBot="1">
       <c r="C14" s="93"/>
       <c r="D14" s="23" t="s">
         <v>65</v>
@@ -14922,7 +15059,7 @@
       <c r="H16" s="30"/>
       <c r="I16" s="31"/>
     </row>
-    <row r="17" spans="3:12" ht="15.75" thickBot="1">
+    <row r="17" spans="3:12" ht="15" thickBot="1">
       <c r="C17" s="94"/>
       <c r="D17" s="32"/>
       <c r="E17" s="33" t="s">
@@ -14933,7 +15070,7 @@
       <c r="H17" s="30"/>
       <c r="I17" s="31"/>
     </row>
-    <row r="18" spans="3:12" ht="15.75" thickBot="1">
+    <row r="18" spans="3:12" ht="15" thickBot="1">
       <c r="C18" s="37" t="s">
         <v>79</v>
       </c>
@@ -14953,7 +15090,7 @@
       <c r="K18" s="24"/>
       <c r="L18" s="25"/>
     </row>
-    <row r="19" spans="3:12" ht="15.75" thickBot="1">
+    <row r="19" spans="3:12" ht="15" thickBot="1">
       <c r="C19" s="92" t="s">
         <v>78</v>
       </c>
@@ -14973,7 +15110,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="21" spans="3:12" ht="15.75" thickBot="1">
+    <row r="21" spans="3:12" ht="15" thickBot="1">
       <c r="C21" s="94"/>
       <c r="D21" s="32"/>
       <c r="E21" s="40" t="s">
@@ -15087,10 +15224,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:V102"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="13" max="13" width="4.85546875" customWidth="1"/>
+    <col min="13" max="13" width="4.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3">
@@ -15605,7 +15742,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:D32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:3">
       <c r="B2" s="6" t="s">
@@ -15728,10 +15865,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:H90"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4">
@@ -16097,9 +16234,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:Z40"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:26">

</xml_diff>

<commit_message>
AnhDXH hoc chu nhat 11/10
</commit_message>
<xml_diff>
--- a/Study_CL.xlsx
+++ b/Study_CL.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" firstSheet="2" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="Knowhow" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,8 @@
     <sheet name="#12" sheetId="14" r:id="rId14"/>
     <sheet name="#13" sheetId="17" r:id="rId15"/>
     <sheet name="#14" sheetId="12" r:id="rId16"/>
-    <sheet name="#16" sheetId="15" r:id="rId17"/>
+    <sheet name="#15" sheetId="18" r:id="rId17"/>
+    <sheet name="#16" sheetId="15" r:id="rId18"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="699">
   <si>
     <t>No.</t>
   </si>
@@ -3745,15 +3746,6 @@
   </si>
   <si>
     <t>Sự khác biệt giữa virtual, pure virtual và override</t>
-  </si>
-  <si>
-    <t>What happens if a base class destructor is not virtual?</t>
-  </si>
-  <si>
-    <t>Can constructors be virtual?</t>
-  </si>
-  <si>
-    <t>What is slicing in C++?</t>
   </si>
   <si>
     <t>#17</t>
@@ -4116,9 +4108,6 @@
     <t>Tăng trước khi dùng</t>
   </si>
   <si>
-    <t>Cấp phát động trong C và C++ (new và malloc)</t>
-  </si>
-  <si>
     <t>Ví dụ :</t>
   </si>
   <si>
@@ -5232,13 +5221,1420 @@
   </si>
   <si>
     <t>Mục đích : Thay đổi hành vi của class cha</t>
+  </si>
+  <si>
+    <t>Virture :</t>
+  </si>
+  <si>
+    <t>Cho phép hàm trong lớp cơ sở được ghi đè bởi hàm trong lớp dẫn xuất (khi kết hợp với override). Nếu không có</t>
+  </si>
+  <si>
+    <t>virture, tại thời điểm compile-time, chương trình sẽ chạy theo con trỏ trỏ đến hàm của lớp cơ sở. Nếu virture,</t>
+  </si>
+  <si>
+    <t>chương trình sẽ trỏ đến đúng đối tượng hàm chỉ định của lớp dẫn xuất</t>
+  </si>
+  <si>
+    <t>Chú ý : Virture được viết ở hàm cơ sở, để chỉ ra rằng nó có thể mang hình thái khác ở lớp dẫn xuất</t>
+  </si>
+  <si>
+    <t>Pure Virtual :</t>
+  </si>
+  <si>
+    <t>Được khai báo trong lớp cơ sở, nó là hàm ảo thuần túy, để bắt buộc chương trình phải mang triển khai phương</t>
+  </si>
+  <si>
+    <t>thức ở lớp dẫn xuất và không thể chạy trực tiếp hàm ở lớp cơ sở.</t>
+  </si>
+  <si>
+    <t>class Animal{</t>
+  </si>
+  <si>
+    <t>};</t>
+  </si>
+  <si>
+    <t>class Cat{</t>
+  </si>
+  <si>
+    <t>virture void sound() = 0</t>
+  </si>
+  <si>
+    <t>void sound(){ printf("Meow");}</t>
+  </si>
+  <si>
+    <t>virture void sound() { printf("Make sound");}</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*class có </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>toàn bộ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> function là pure virture function được gọi là </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>interface class</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>*class có</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ít nhất 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pure virtual function được gọi là class trừu tượng ( </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>abstract class</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>Ví dụ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        cout &lt;&lt; "Woof!\n";</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>void speak() override {</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> // Compiler kiểm tra có override hợp lệ không</t>
+    </r>
+  </si>
+  <si>
+    <t>Hàm constructor có thể trở thành virtual không ?</t>
+  </si>
+  <si>
+    <t>Điều gì sẽ xảy ra khi hàm hủy (destructor) của class base không phải là virtual ?</t>
+  </si>
+  <si>
+    <t>Slicing trong C++ là gì? Khi khai báo class dẫn xuất theo kiểu cấp phát động, kiểu con trỏ cha, thì những phương thức, thuộc tính mới của class con có chỗ để chứa trong con trỏ đó không ? Cơ chế là gì ? Tại sao ?</t>
+  </si>
+  <si>
+    <t>Sẽ gây rò rỉ bộ nhớ (Memory Leak) khi thực hiện xóa class con.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">dẫn đến </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>rò rỉ bộ nhớ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> và rủi ro lỗi </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>undefined behavior</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Khi xóa đối tượng đó, chương trình chỉ gọi đến </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>destructor tương ứng với kiểu con trỏ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, dẫn đến </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>destructor của lớp deliveried không được gọi</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cách làm đúng và an toàn : thêm virtual vào cho hàm hủy của class cơ sở, khi gọi hàm hủy, chương trình sẽ gọi từ destructor của </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>class dẫn xuất -&gt; class cơ sở</t>
+    </r>
+  </si>
+  <si>
+    <t>class Base {</t>
+  </si>
+  <si>
+    <t>public:</t>
+  </si>
+  <si>
+    <t>class Derived : public Base {</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ~Derived() {</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    virtual ~Base() {</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>KHÔNG THỂ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, và </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C++ cấm hoàn toàn</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> việc khai báo constructor là virtual.</t>
+    </r>
+  </si>
+  <si>
+    <t>nếu gọi vào virtual constructor -&gt; chương trình sẽ tra vtable pointer -&gt; Không có do constructor chưa thực thi xong -&gt; Vòng lặp luẩn quẩn</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Lý do là </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>để gọi 1 virtual function</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> thì </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>cần vtable pointer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, mà </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vtable chỉ được khởi tạo khi constructor của đối tượng thực thi xong</t>
+    </r>
+  </si>
+  <si>
+    <t>sử dụng nó nữa, hệ thống sẽ tự động clean up đối tượng đó để tránh các vấn đề về bộ nhớ, lãng phí tài nguyên</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cơ chế hoạt động</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của RAII</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Constructor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Cấp phát tài nguyên lúc khởi tạo</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>RAII là gì (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Resource Acquisition Is Initialization</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Destructor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : Dọn dẹp sạch tài nguyên khi đối tượng ra khỏi scope</t>
+    </r>
+  </si>
+  <si>
+    <t>Một số mô hình RAII trong C++</t>
+  </si>
+  <si>
+    <t>Bộ nhớ động :</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>Tự đóng file khi bị hủy</t>
+  </si>
+  <si>
+    <t>Mutex</t>
+  </si>
+  <si>
+    <t>std::fstream :</t>
+  </si>
+  <si>
+    <t>std::unique_ptr , std::shared_ptr, std::vector : Tự động giải phóng khi hết scope</t>
+  </si>
+  <si>
+    <t>std::lock_guard, std::unique_lock : tự động unlock khi scope kết thúc</t>
+  </si>
+  <si>
+    <r>
+      <t>Khái niệm : Dịch ra là "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Tài nguyên được cấp phát lúc khởi tạo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">". Tức là nếu </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gói gọn tài nguyên trong 1 object</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, khi không </t>
+    </r>
+  </si>
+  <si>
+    <t>Cấp phát động trong C và C++</t>
+  </si>
+  <si>
+    <t>Cấp phát động trong C và C++
+Trong C : malloc(), calloc(), realloc(), free()
+Trong C++ : new()</t>
+  </si>
+  <si>
+    <t>Trong C :</t>
+  </si>
+  <si>
+    <t>malloc()</t>
+  </si>
+  <si>
+    <t>calloc()</t>
+  </si>
+  <si>
+    <t>realloc()</t>
+  </si>
+  <si>
+    <t>Cú pháp :</t>
+  </si>
+  <si>
+    <r>
+      <t>int* arr = (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>int*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>malloc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>n *</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sizeof(int))</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>int*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : malloc sẽ trả về kiểu void* nên cần ép kiểu cho nó</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>n</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : thường thì biến số n không cố định sẽ được nhân với </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sizeof</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(kiểu kích thước) để cấp phát kích thước mong muốn</t>
+    </r>
+  </si>
+  <si>
+    <t>Khi khởi tạo, các giá trị ban đầu là rác</t>
+  </si>
+  <si>
+    <t>Giống hệt malloc về cách dùng, chỉ khác là thay vì truyền vào tổng byte thì truyền vào số phần tử và kích thước. Giá trị khởi tạo ban đầu cho các phần tử được set = 0</t>
+  </si>
+  <si>
+    <r>
+      <t>int* arr = (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>int*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>calloc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(element_num </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>n ,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> size_each </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Q</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>int*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : calloc sẽ trả về kiểu void* nên cần ép kiểu cho nó</t>
+    </r>
+  </si>
+  <si>
+    <t>size của dữ liệu = n*Q</t>
+  </si>
+  <si>
+    <t>* Dùng calloc để tránh quên khởi tạo giá trị ban đầu cho dữ liệu, hoặc muốn ban đầu tất cả = 0</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dùng để </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>thay đổi kích thước</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (tăng hoặc giảm) 1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>con trỏ đã được cấp phát động</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> bằng malloc(), calloc(), realloc() và </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>không làm thay đổi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> các phần tử cũ trong con trỏ đó</t>
+    </r>
+  </si>
+  <si>
+    <t>Có 2 trường hợp khi dùng realloc() :</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mở rộng tại chỗ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> khi vẫn còn </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>đủ chỗ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> trong vùng nhớ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Nếu </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vùng nhớ không đủ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, realloc sẽ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>copy toàn bộ phần tử cũ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sang </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vùng nhớ mới</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> có </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>đủ không gian</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> để mở rộng, rồi </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>giải phóng vùng nhớ cũ.</t>
+    </r>
+  </si>
+  <si>
+    <t>int *arr = (int*)malloc(3 * sizeof(int));</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>arr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>int*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>realloc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>arr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5 * sizeof(int)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">// đối số của realloc ( </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>đối tượng con trỏ cần thay đổi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dung lượng sau khi thay đổi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> )</t>
+    </r>
+  </si>
+  <si>
+    <t>free(ptr)</t>
+  </si>
+  <si>
+    <t>Cách dùng đúng</t>
+  </si>
+  <si>
+    <t>free(ptr);</t>
+  </si>
+  <si>
+    <t>ptr = NULL;</t>
+  </si>
+  <si>
+    <r>
+      <t>Bản chất là delete con trỏ ptr, nhưng lúc này nếu</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> gọi lại </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>biến</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ptr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> thì nó đang là </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dangling pointer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, sẽ dẫn đến lỗi </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>undefined behavior</t>
+    </r>
+  </si>
+  <si>
+    <t>Trong C++ :</t>
+  </si>
+  <si>
+    <t>new() và delete</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Được sinh ra để </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>cấp phát động cho class</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> vì </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>malloc không có cơ chế hỗ trợ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> cho </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>contructor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> và </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>destructor</t>
+    </r>
+  </si>
+  <si>
+    <t>new()</t>
+  </si>
+  <si>
+    <t>cú pháp :</t>
+  </si>
+  <si>
+    <t>khai báo biến :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">khai báo mảng : </t>
+  </si>
+  <si>
+    <t>khai báo class :</t>
+  </si>
+  <si>
+    <t>int* p = new int(10);</t>
+  </si>
+  <si>
+    <t>int* arr = new int[3];</t>
+  </si>
+  <si>
+    <t>// cấp phát 1 mảng có 3 phần tử</t>
+  </si>
+  <si>
+    <t>// cấp phát động 1 biến int mang giá trị 10</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Printer* p = new Printer( </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>đối số của constructor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>copy constructor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) ;</t>
+    </r>
+  </si>
+  <si>
+    <t>delete()</t>
+  </si>
+  <si>
+    <t>clear biến :</t>
+  </si>
+  <si>
+    <t>delete p;</t>
+  </si>
+  <si>
+    <t>delete arr[];</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5394,6 +6790,20 @@
       <color rgb="FFD4D4D4"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="16">
@@ -5681,7 +7091,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -5873,6 +7283,9 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -11342,72 +12755,72 @@
     </row>
     <row r="3" spans="2:5">
       <c r="C3" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" spans="2:5">
       <c r="C5" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="D6" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="E6" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="D7" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="E7" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="C9" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="11" spans="2:5">
       <c r="C11" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="D12" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="C15" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
     </row>
     <row r="17" spans="3:19">
       <c r="D17" s="83" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="E17" s="87"/>
       <c r="F17" s="87"/>
       <c r="G17" s="87"/>
       <c r="H17" s="87"/>
       <c r="I17" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
     </row>
     <row r="18" spans="3:19">
       <c r="D18" s="83" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="E18" s="87"/>
       <c r="F18" s="87"/>
       <c r="G18" s="87"/>
       <c r="H18" s="87"/>
       <c r="I18" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
     </row>
     <row r="19" spans="3:19">
@@ -11419,31 +12832,31 @@
     </row>
     <row r="20" spans="3:19">
       <c r="D20" s="85" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="E20" s="87"/>
       <c r="F20" s="87"/>
       <c r="G20" s="87"/>
       <c r="H20" s="87"/>
       <c r="I20" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
     </row>
     <row r="21" spans="3:19">
       <c r="D21" s="86" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="E21" s="87"/>
       <c r="F21" s="87"/>
       <c r="G21" s="87"/>
       <c r="H21" s="87"/>
       <c r="I21" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
     </row>
     <row r="22" spans="3:19">
       <c r="D22" s="86" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="E22" s="87"/>
       <c r="F22" s="87"/>
@@ -11468,7 +12881,7 @@
     </row>
     <row r="25" spans="3:19">
       <c r="D25" s="85" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="E25" s="87"/>
       <c r="F25" s="87"/>
@@ -11477,7 +12890,7 @@
     </row>
     <row r="26" spans="3:19">
       <c r="D26" s="86" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
       <c r="E26" s="87"/>
       <c r="F26" s="87"/>
@@ -11486,7 +12899,7 @@
     </row>
     <row r="27" spans="3:19">
       <c r="D27" s="86" t="s">
-        <v>560</v>
+        <v>556</v>
       </c>
       <c r="E27" s="87"/>
       <c r="F27" s="87"/>
@@ -11504,7 +12917,7 @@
     </row>
     <row r="31" spans="3:19">
       <c r="C31" s="88" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="D31" s="88"/>
       <c r="E31" s="88"/>
@@ -11516,7 +12929,7 @@
       <c r="K31" s="88"/>
       <c r="L31" s="88"/>
       <c r="M31" s="89" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="N31" s="89"/>
       <c r="O31" s="89"/>
@@ -11547,7 +12960,7 @@
     <row r="33" spans="3:19">
       <c r="C33" s="88"/>
       <c r="D33" s="88" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="E33" s="88"/>
       <c r="F33" s="88"/>
@@ -11558,7 +12971,7 @@
       <c r="K33" s="88"/>
       <c r="L33" s="88"/>
       <c r="M33" s="89" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="N33" s="89"/>
       <c r="O33" s="89"/>
@@ -11579,7 +12992,7 @@
       <c r="K34" s="88"/>
       <c r="L34" s="88"/>
       <c r="M34" s="89" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="N34" s="89"/>
       <c r="O34" s="89"/>
@@ -11612,7 +13025,7 @@
     <row r="36" spans="3:19">
       <c r="C36" s="88"/>
       <c r="D36" s="88" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="E36" s="88"/>
       <c r="F36" s="88"/>
@@ -11626,7 +13039,7 @@
     <row r="37" spans="3:19">
       <c r="C37" s="88"/>
       <c r="D37" s="88" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="E37" s="88"/>
       <c r="F37" s="88"/>
@@ -11664,101 +13077,101 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="C4" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="D6" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="D7" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="D8" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="E8" s="80"/>
     </row>
     <row r="9" spans="2:5">
       <c r="D9" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="D10" t="s">
-        <v>540</v>
+        <v>536</v>
       </c>
     </row>
     <row r="11" spans="2:5">
       <c r="D11" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="D12" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="D13" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
     </row>
     <row r="14" spans="2:5">
       <c r="D14" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="D15" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="D16" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
     </row>
     <row r="17" spans="3:12">
       <c r="D17" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
     </row>
     <row r="18" spans="3:12">
       <c r="D18" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
     </row>
     <row r="19" spans="3:12">
       <c r="D19" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
     </row>
     <row r="22" spans="3:12">
       <c r="C22" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
     </row>
     <row r="23" spans="3:12">
       <c r="D23" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="L23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
     </row>
     <row r="24" spans="3:12">
       <c r="D24" s="81" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="E24" s="90"/>
       <c r="F24" s="90"/>
@@ -11769,7 +13182,7 @@
     </row>
     <row r="25" spans="3:12">
       <c r="D25" s="81" t="s">
-        <v>577</v>
+        <v>573</v>
       </c>
       <c r="E25" s="90"/>
       <c r="F25" s="90"/>
@@ -11780,12 +13193,12 @@
     </row>
     <row r="27" spans="3:12">
       <c r="D27" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
     </row>
     <row r="28" spans="3:12">
       <c r="D28" s="81" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="E28" s="90"/>
       <c r="F28" s="90"/>
@@ -11796,7 +13209,7 @@
     </row>
     <row r="29" spans="3:12">
       <c r="D29" s="81" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="E29" s="90"/>
       <c r="F29" s="90"/>
@@ -11807,7 +13220,7 @@
     </row>
     <row r="30" spans="3:12">
       <c r="D30" s="82" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="E30" s="90"/>
       <c r="F30" s="90"/>
@@ -11818,42 +13231,42 @@
     </row>
     <row r="33" spans="3:13">
       <c r="D33" s="91" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
     </row>
     <row r="34" spans="3:13">
       <c r="E34" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
     </row>
     <row r="35" spans="3:13">
       <c r="F35" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
     </row>
     <row r="36" spans="3:13">
       <c r="F36" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
     </row>
     <row r="39" spans="3:13">
       <c r="C39" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
     </row>
     <row r="41" spans="3:13">
       <c r="D41" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
     </row>
     <row r="43" spans="3:13">
       <c r="D43" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
     </row>
     <row r="44" spans="3:13">
       <c r="E44" s="81" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="F44" s="90"/>
       <c r="G44" s="90"/>
@@ -11877,7 +13290,7 @@
     </row>
     <row r="46" spans="3:13">
       <c r="E46" s="81" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="F46" s="90"/>
       <c r="G46" s="90"/>
@@ -11890,7 +13303,7 @@
     </row>
     <row r="47" spans="3:13">
       <c r="E47" s="81" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="F47" s="90"/>
       <c r="G47" s="90"/>
@@ -11903,7 +13316,7 @@
     </row>
     <row r="48" spans="3:13">
       <c r="E48" s="81" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="F48" s="90"/>
       <c r="G48" s="90"/>
@@ -11916,7 +13329,7 @@
     </row>
     <row r="49" spans="4:13">
       <c r="E49" s="82" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="F49" s="90"/>
       <c r="G49" s="90"/>
@@ -11929,7 +13342,7 @@
     </row>
     <row r="50" spans="4:13">
       <c r="E50" s="81" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="F50" s="90"/>
       <c r="G50" s="90"/>
@@ -11942,27 +13355,27 @@
     </row>
     <row r="53" spans="4:13">
       <c r="D53" s="91" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
     </row>
     <row r="54" spans="4:13">
       <c r="E54" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
     </row>
     <row r="55" spans="4:13">
       <c r="E55" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
     </row>
     <row r="56" spans="4:13">
       <c r="E56" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
     </row>
     <row r="57" spans="4:13">
       <c r="E57" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
     </row>
   </sheetData>
@@ -11978,89 +13391,89 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
     </row>
     <row r="3" spans="2:5">
       <c r="C3" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="D3" t="s">
+        <v>508</v>
+      </c>
+      <c r="E3" t="s">
         <v>511</v>
-      </c>
-      <c r="E3" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="C4" s="80" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="D4" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="E4" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="C7" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="C8" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="C10" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
     </row>
     <row r="11" spans="2:5">
       <c r="C11" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="C12" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="C13" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
     </row>
     <row r="14" spans="2:5">
       <c r="C14" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="C15" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="C16" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
     </row>
     <row r="21" spans="3:3">
@@ -12070,17 +13483,17 @@
     </row>
     <row r="23" spans="3:3">
       <c r="C23" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" t="s">
-        <v>530</v>
+        <v>526</v>
       </c>
     </row>
     <row r="25" spans="3:3">
       <c r="C25" t="s">
-        <v>531</v>
+        <v>527</v>
       </c>
     </row>
   </sheetData>
@@ -12090,12 +13503,75 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2"/>
+  <dimension ref="B2:E16"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
-        <v>439</v>
+        <v>643</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="C3" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="C4" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="C6" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="D7" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="D8" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5">
+      <c r="C10" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5">
+      <c r="C11" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5">
+      <c r="D12" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="C13" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5">
+      <c r="D14" t="s">
+        <v>650</v>
+      </c>
+      <c r="E14" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5">
+      <c r="C15" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5">
+      <c r="D16" t="s">
+        <v>652</v>
       </c>
     </row>
   </sheetData>
@@ -12152,86 +13628,565 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:D20"/>
+  <dimension ref="B2:I48"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:4">
       <c r="B2" s="6" t="s">
-        <v>480</v>
+        <v>654</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" ht="18.5">
+      <c r="C3" s="96" t="s">
+        <v>656</v>
+      </c>
+      <c r="D3" s="97"/>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="C5" t="s">
+        <v>657</v>
+      </c>
+      <c r="D5" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="D6" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="D7" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="D8" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="D9" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4">
+      <c r="C11" t="s">
+        <v>658</v>
+      </c>
+      <c r="D11" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4">
+      <c r="D12" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="D13" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="D14" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4">
+      <c r="D15" s="95" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="D16" s="76" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5">
+      <c r="C17" t="s">
+        <v>659</v>
+      </c>
+      <c r="D17" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5">
+      <c r="D18" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5">
+      <c r="E19" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5">
+      <c r="E20" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="21" spans="3:5">
+      <c r="D21" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="22" spans="3:5">
+      <c r="D22" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="23" spans="3:5">
+      <c r="D23" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5">
+      <c r="D24" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="26" spans="3:5">
+      <c r="C26" t="s">
+        <v>677</v>
+      </c>
+      <c r="D26" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="27" spans="3:5">
+      <c r="D27" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="28" spans="3:5">
+      <c r="E28" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="29" spans="3:5">
+      <c r="E29" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="33" spans="3:9" ht="18.5">
+      <c r="C33" s="96" t="s">
+        <v>682</v>
+      </c>
+      <c r="D33" s="97"/>
+    </row>
+    <row r="35" spans="3:9">
+      <c r="C35" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="36" spans="3:9">
+      <c r="D36" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="38" spans="3:9">
+      <c r="D38" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="39" spans="3:9">
+      <c r="E39" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="40" spans="3:9">
+      <c r="E40" t="s">
+        <v>687</v>
+      </c>
+      <c r="G40" t="s">
+        <v>690</v>
+      </c>
+      <c r="I40" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="41" spans="3:9">
+      <c r="E41" t="s">
+        <v>688</v>
+      </c>
+      <c r="G41" t="s">
+        <v>691</v>
+      </c>
+      <c r="I41" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="42" spans="3:9">
+      <c r="E42" t="s">
+        <v>689</v>
+      </c>
+      <c r="G42" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="44" spans="3:9">
+      <c r="D44" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="45" spans="3:9">
+      <c r="E45" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="46" spans="3:9">
+      <c r="E46" t="s">
+        <v>696</v>
+      </c>
+      <c r="G46" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="47" spans="3:9">
+      <c r="E47" t="s">
+        <v>688</v>
+      </c>
+      <c r="G47" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="48" spans="3:9">
+      <c r="E48" t="s">
+        <v>689</v>
+      </c>
+      <c r="G48" t="s">
+        <v>697</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:E85"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="B2" s="6" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="3" spans="2:4">
       <c r="C3" t="s">
+        <v>528</v>
+      </c>
+      <c r="D3" t="s">
         <v>532</v>
-      </c>
-      <c r="D3" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="4" spans="2:4">
       <c r="C4" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="D4" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5" spans="2:4">
       <c r="C5" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="D5" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
     </row>
     <row r="10" spans="2:4">
       <c r="B10" s="6" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="11" spans="2:4">
       <c r="C11" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
     </row>
     <row r="12" spans="2:4">
       <c r="C12" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
     </row>
     <row r="13" spans="2:4">
       <c r="C13" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
     </row>
     <row r="14" spans="2:4">
       <c r="C14" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
     </row>
     <row r="16" spans="2:4">
       <c r="C16" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="C17" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="C18" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="C19" t="s">
         <v>603</v>
       </c>
     </row>
-    <row r="17" spans="3:3">
-      <c r="C17" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="18" spans="3:3">
-      <c r="C18" t="s">
+    <row r="20" spans="2:5">
+      <c r="C20" t="s">
         <v>605</v>
       </c>
     </row>
-    <row r="19" spans="3:3">
-      <c r="C19" t="s">
+    <row r="22" spans="2:5">
+      <c r="D22" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="E23" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="E24" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="E25" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5">
+      <c r="B28" s="6" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5">
+      <c r="C29" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5">
+      <c r="D30" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="20" spans="3:3">
-      <c r="C20" t="s">
+    <row r="31" spans="2:5">
+      <c r="D31" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5">
+      <c r="D32" t="s">
         <v>609</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5">
+      <c r="D34" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5">
+      <c r="D36" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="37" spans="3:5">
+      <c r="E37" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5">
+      <c r="E38" s="17" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5">
+      <c r="E39" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="41" spans="3:5">
+      <c r="E41" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5">
+      <c r="E42" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="43" spans="3:5">
+      <c r="E43" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="45" spans="3:5">
+      <c r="C45" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="46" spans="3:5">
+      <c r="D46" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="47" spans="3:5">
+      <c r="D47" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5">
+      <c r="D49" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5">
+      <c r="E50" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5">
+      <c r="E51" s="17" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5">
+      <c r="E52" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5">
+      <c r="E54" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5">
+      <c r="E55" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5">
+      <c r="E56" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5">
+      <c r="D58" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5">
+      <c r="D59" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5">
+      <c r="B62" s="6" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5">
+      <c r="C63" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5">
+      <c r="C64" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="65" spans="3:4">
+      <c r="C65" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4">
+      <c r="C67" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="69" spans="3:4">
+      <c r="D69" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="70" spans="3:4">
+      <c r="D70" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="71" spans="3:4">
+      <c r="D71" s="17" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="72" spans="3:4">
+      <c r="D72" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="73" spans="3:4">
+      <c r="D73" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="75" spans="3:4">
+      <c r="D75" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="76" spans="3:4">
+      <c r="D76" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="77" spans="3:4">
+      <c r="D77" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="78" spans="3:4">
+      <c r="D78" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="79" spans="3:4">
+      <c r="D79" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="82" spans="2:3">
+      <c r="B82" s="6" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="83" spans="2:3">
+      <c r="C83" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="84" spans="2:3">
+      <c r="C84" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="85" spans="2:3">
+      <c r="C85" t="s">
+        <v>638</v>
       </c>
     </row>
   </sheetData>
@@ -14128,7 +16083,7 @@
         <v>287</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="D49" s="51">
         <v>0.9</v>
@@ -14143,7 +16098,7 @@
         <v>319</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="D50" s="42">
         <v>1</v>
@@ -14171,7 +16126,7 @@
         <v>321</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="D52" s="42">
         <v>1</v>
@@ -14188,7 +16143,9 @@
       <c r="C53" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="D53" s="6"/>
+      <c r="D53" s="42">
+        <v>1</v>
+      </c>
       <c r="E53" s="6"/>
       <c r="F53" s="16" t="s">
         <v>14</v>
@@ -14209,16 +16166,20 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="2:6">
+    <row r="55" spans="2:6" ht="43.5">
       <c r="B55" s="5" t="s">
         <v>448</v>
       </c>
-      <c r="C55" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="D55" s="6"/>
+      <c r="C55" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="D55" s="51">
+        <v>0.5</v>
+      </c>
       <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
+      <c r="F55" s="16" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="56" spans="2:6">
       <c r="B56" s="5" t="s">
@@ -14227,9 +16188,11 @@
       <c r="C56" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="D56" s="6"/>
+      <c r="D56" s="42">
+        <v>0.5</v>
+      </c>
       <c r="E56" s="16" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="F56" s="6"/>
     </row>
@@ -14238,7 +16201,7 @@
         <v>16.100000000000001</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="D57" s="42">
         <v>1</v>
@@ -14253,7 +16216,7 @@
         <v>16.2</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="D58" s="42">
         <v>1</v>
@@ -14270,38 +16233,50 @@
       <c r="C59" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="D59" s="6"/>
+      <c r="D59" s="42">
+        <v>1</v>
+      </c>
       <c r="E59" s="6"/>
-      <c r="F59" s="6"/>
-    </row>
-    <row r="60" spans="2:6">
+      <c r="F59" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" ht="29">
       <c r="B60" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="C60" s="6" t="s">
-        <v>452</v>
-      </c>
-      <c r="D60" s="6"/>
+      <c r="C60" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="D60" s="42">
+        <v>1</v>
+      </c>
       <c r="E60" s="6"/>
-      <c r="F60" s="6"/>
+      <c r="F60" s="16" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="61" spans="2:6">
       <c r="B61" s="5">
         <v>16.5</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>453</v>
-      </c>
-      <c r="D61" s="6"/>
+        <v>625</v>
+      </c>
+      <c r="D61" s="42">
+        <v>1</v>
+      </c>
       <c r="E61" s="6"/>
-      <c r="F61" s="6"/>
-    </row>
-    <row r="62" spans="2:6">
+      <c r="F61" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" ht="58">
       <c r="B62" s="5">
         <v>16.600000000000001</v>
       </c>
-      <c r="C62" s="6" t="s">
-        <v>454</v>
+      <c r="C62" s="7" t="s">
+        <v>627</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
@@ -14312,7 +16287,7 @@
         <v>16.7</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
@@ -14320,10 +16295,10 @@
     </row>
     <row r="64" spans="2:6">
       <c r="B64" s="5" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
@@ -14334,7 +16309,7 @@
         <v>17.100000000000001</v>
       </c>
       <c r="C65" s="78" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
@@ -14345,7 +16320,7 @@
         <v>17.2</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
@@ -14356,11 +16331,11 @@
         <v>17.3</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="16" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="F67" s="6"/>
     </row>
@@ -14369,7 +16344,7 @@
         <v>17.399999999999999</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
@@ -14380,7 +16355,7 @@
         <v>17.5</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
@@ -14388,10 +16363,10 @@
     </row>
     <row r="70" spans="2:6">
       <c r="B70" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="C70" s="6" t="s">
         <v>460</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>463</v>
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
@@ -14402,7 +16377,7 @@
         <v>18.100000000000001</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
@@ -14413,7 +16388,7 @@
         <v>18.2</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
@@ -14424,7 +16399,7 @@
         <v>18.3</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
@@ -14435,7 +16410,7 @@
         <v>18.399999999999999</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
@@ -14443,10 +16418,10 @@
     </row>
     <row r="75" spans="2:6">
       <c r="B75" s="5" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
@@ -14457,7 +16432,7 @@
         <v>19.100000000000001</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
@@ -14465,7 +16440,7 @@
     </row>
     <row r="77" spans="2:6">
       <c r="B77" s="5" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>438</v>
@@ -14476,7 +16451,7 @@
     </row>
     <row r="78" spans="2:6">
       <c r="B78" s="5" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>288</v>
@@ -14501,7 +16476,7 @@
         <v>21.2</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
@@ -14509,36 +16484,36 @@
     </row>
     <row r="81" spans="2:6">
       <c r="B81" s="5" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="C81" s="6" t="s">
         <v>323</v>
       </c>
       <c r="D81" s="6"/>
       <c r="E81" s="16" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F81" s="6"/>
     </row>
     <row r="82" spans="2:6">
       <c r="B82" s="5" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="D82" s="6"/>
       <c r="E82" s="16" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F82" s="6"/>
     </row>
     <row r="83" spans="2:6">
       <c r="B83" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="C83" s="6" t="s">
         <v>481</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>484</v>
       </c>
       <c r="D83" s="6"/>
       <c r="E83" s="16"/>
@@ -14546,10 +16521,10 @@
     </row>
     <row r="84" spans="2:6">
       <c r="B84" s="5" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D84" s="6"/>
       <c r="E84" s="16"/>
@@ -14557,23 +16532,23 @@
     </row>
     <row r="85" spans="2:6" ht="58">
       <c r="B85" s="5" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="C85" s="79" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D85" s="6"/>
       <c r="E85" s="16" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="F85" s="6"/>
     </row>
     <row r="86" spans="2:6" ht="29">
       <c r="B86" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="16"/>
@@ -14581,10 +16556,10 @@
     </row>
     <row r="87" spans="2:6">
       <c r="B87" s="5" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D87" s="6"/>
       <c r="E87" s="16"/>
@@ -14592,10 +16567,10 @@
     </row>
     <row r="88" spans="2:6" ht="58">
       <c r="B88" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="D88" s="6"/>
       <c r="E88" s="16"/>
@@ -14603,10 +16578,10 @@
     </row>
     <row r="89" spans="2:6" ht="29">
       <c r="B89" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D89" s="6"/>
       <c r="E89" s="16"/>
@@ -14614,14 +16589,14 @@
     </row>
     <row r="90" spans="2:6">
       <c r="B90" s="77" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="C90" s="57" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="D90" s="1"/>
       <c r="E90" s="49" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="F90" s="1"/>
     </row>
@@ -14684,6 +16659,10 @@
     <hyperlink ref="F50" location="'#10'!B2" display="Link"/>
     <hyperlink ref="F53" location="'#13'!B2" display="Link"/>
     <hyperlink ref="F58" location="'#16'!B10" display="Link"/>
+    <hyperlink ref="F59" location="'#16'!B28" display="Link"/>
+    <hyperlink ref="F60" location="'#16'!B62" display="Link"/>
+    <hyperlink ref="F61" location="'#16'!B82" display="Link"/>
+    <hyperlink ref="F55" location="'#15'!B2" display="Link"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId12"/>

</xml_diff>

<commit_message>
AnhDXH day file 11242025
</commit_message>
<xml_diff>
--- a/Study_CL.xlsx
+++ b/Study_CL.xlsx
@@ -29,16 +29,17 @@
     <sheet name="#17" sheetId="32" r:id="rId20"/>
     <sheet name="#19" sheetId="22" r:id="rId21"/>
     <sheet name="#20" sheetId="27" r:id="rId22"/>
-    <sheet name="#23" sheetId="30" r:id="rId23"/>
-    <sheet name="#24" sheetId="20" r:id="rId24"/>
-    <sheet name="#25" sheetId="21" r:id="rId25"/>
-    <sheet name="#26" sheetId="28" r:id="rId26"/>
-    <sheet name="#27" sheetId="31" r:id="rId27"/>
-    <sheet name="#28" sheetId="29" r:id="rId28"/>
-    <sheet name="#29" sheetId="23" r:id="rId29"/>
-    <sheet name="#30" sheetId="24" r:id="rId30"/>
-    <sheet name="#31" sheetId="19" r:id="rId31"/>
-    <sheet name="#32" sheetId="25" r:id="rId32"/>
+    <sheet name="#21" sheetId="33" r:id="rId23"/>
+    <sheet name="#23" sheetId="30" r:id="rId24"/>
+    <sheet name="#24" sheetId="20" r:id="rId25"/>
+    <sheet name="#25" sheetId="21" r:id="rId26"/>
+    <sheet name="#26" sheetId="28" r:id="rId27"/>
+    <sheet name="#27" sheetId="31" r:id="rId28"/>
+    <sheet name="#28" sheetId="29" r:id="rId29"/>
+    <sheet name="#29" sheetId="23" r:id="rId30"/>
+    <sheet name="#30" sheetId="24" r:id="rId31"/>
+    <sheet name="#31" sheetId="19" r:id="rId32"/>
+    <sheet name="#32" sheetId="25" r:id="rId33"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="1017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1392" uniqueCount="1044">
   <si>
     <t>No.</t>
   </si>
@@ -13129,13 +13130,152 @@
   </si>
   <si>
     <t>#include &lt;algorithm&gt;</t>
+  </si>
+  <si>
+    <t>21.10</t>
+  </si>
+  <si>
+    <t>21.11</t>
+  </si>
+  <si>
+    <t>21.12</t>
+  </si>
+  <si>
+    <t>#33</t>
+  </si>
+  <si>
+    <t>Các loại thư viện</t>
+  </si>
+  <si>
+    <t>Shared Library</t>
+  </si>
+  <si>
+    <t>Static Library</t>
+  </si>
+  <si>
+    <t>Header-only Library</t>
+  </si>
+  <si>
+    <t>std::mutex mtx;</t>
+  </si>
+  <si>
+    <t>Khóa mutex</t>
+  </si>
+  <si>
+    <t>std::mutex mtx;  // Sẽ ra sao nếu chỉ lock mutex mà quên không unlock</t>
+  </si>
+  <si>
+    <t>Khái niệm : là một cơ chế giúp đảm bảo chỉ một thread được truy cập tài nguyên chung tại cùng một thời điểm.</t>
+  </si>
+  <si>
+    <t>// khai báo thư viện</t>
+  </si>
+  <si>
+    <t>// khai báo biến mutex là mtx</t>
+  </si>
+  <si>
+    <t>………</t>
+  </si>
+  <si>
+    <t>mtx.lock();</t>
+  </si>
+  <si>
+    <t>mtx.unlock();</t>
+  </si>
+  <si>
+    <t>// tài nguyên chung cần sửa</t>
+  </si>
+  <si>
+    <t>// dùng mutex để khóa</t>
+  </si>
+  <si>
+    <t>// dùng mutex để mở khóa</t>
+  </si>
+  <si>
+    <t>Sẽ ra sao nếu chỉ lock mutex mà quên không unlock</t>
+  </si>
+  <si>
+    <r>
+      <t>#include</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;mutex&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Nếu hoạt động với nhiều thread, thread khác sẽ chờ đợi và không thể giữ được khóa mutex -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Deadlock</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">hoặc nếu gọi lần 2 về chính thread khóa mà lần 1 chưa unlock() -&gt; tự </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Deadlock</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mục đích sử dụng : để </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tránh race condition</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> khi có quá nhiều thread tranh nhau sửa tài nguyên dẫn đến hoạt động sai</t>
+    </r>
+  </si>
+  <si>
+    <t>race condition là gì</t>
+  </si>
+  <si>
+    <t>deadlock là gì ?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -13321,6 +13461,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -13735,7 +13883,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -13964,6 +14112,9 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -14015,9 +14166,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -21214,16 +21363,16 @@
       </c>
     </row>
     <row r="89" spans="2:9" ht="54" customHeight="1">
-      <c r="B89" s="119" t="s">
+      <c r="B89" s="120" t="s">
         <v>618</v>
       </c>
-      <c r="C89" s="120"/>
-      <c r="D89" s="120"/>
-      <c r="E89" s="120"/>
-      <c r="F89" s="120"/>
-      <c r="G89" s="120"/>
-      <c r="H89" s="120"/>
-      <c r="I89" s="120"/>
+      <c r="C89" s="121"/>
+      <c r="D89" s="121"/>
+      <c r="E89" s="121"/>
+      <c r="F89" s="121"/>
+      <c r="G89" s="121"/>
+      <c r="H89" s="121"/>
+      <c r="I89" s="121"/>
     </row>
     <row r="91" spans="2:9">
       <c r="B91" t="s">
@@ -22566,11 +22715,11 @@
     </row>
     <row r="3" spans="2:7" ht="15.75" thickBot="1"/>
     <row r="4" spans="2:7">
-      <c r="C4" s="121" t="s">
+      <c r="C4" s="122" t="s">
         <v>914</v>
       </c>
-      <c r="D4" s="122"/>
-      <c r="E4" s="123"/>
+      <c r="D4" s="123"/>
+      <c r="E4" s="124"/>
       <c r="F4" t="s">
         <v>918</v>
       </c>
@@ -22579,9 +22728,9 @@
       </c>
     </row>
     <row r="5" spans="2:7" ht="15.75" thickBot="1">
-      <c r="C5" s="124"/>
-      <c r="D5" s="125"/>
-      <c r="E5" s="126"/>
+      <c r="C5" s="125"/>
+      <c r="D5" s="126"/>
+      <c r="E5" s="127"/>
       <c r="F5" t="s">
         <v>920</v>
       </c>
@@ -22590,11 +22739,11 @@
       </c>
     </row>
     <row r="6" spans="2:7">
-      <c r="C6" s="121" t="s">
+      <c r="C6" s="122" t="s">
         <v>915</v>
       </c>
-      <c r="D6" s="122"/>
-      <c r="E6" s="123"/>
+      <c r="D6" s="123"/>
+      <c r="E6" s="124"/>
       <c r="F6" t="s">
         <v>918</v>
       </c>
@@ -22603,9 +22752,9 @@
       </c>
     </row>
     <row r="7" spans="2:7" ht="15.75" thickBot="1">
-      <c r="C7" s="124"/>
-      <c r="D7" s="125"/>
-      <c r="E7" s="126"/>
+      <c r="C7" s="125"/>
+      <c r="D7" s="126"/>
+      <c r="E7" s="127"/>
       <c r="F7" t="s">
         <v>920</v>
       </c>
@@ -22614,11 +22763,11 @@
       </c>
     </row>
     <row r="8" spans="2:7">
-      <c r="C8" s="121" t="s">
+      <c r="C8" s="122" t="s">
         <v>916</v>
       </c>
-      <c r="D8" s="122"/>
-      <c r="E8" s="123"/>
+      <c r="D8" s="123"/>
+      <c r="E8" s="124"/>
       <c r="F8" t="s">
         <v>918</v>
       </c>
@@ -22627,9 +22776,9 @@
       </c>
     </row>
     <row r="9" spans="2:7" ht="15.75" thickBot="1">
-      <c r="C9" s="124"/>
-      <c r="D9" s="125"/>
-      <c r="E9" s="126"/>
+      <c r="C9" s="125"/>
+      <c r="D9" s="126"/>
+      <c r="E9" s="127"/>
       <c r="F9" t="s">
         <v>920</v>
       </c>
@@ -22638,11 +22787,11 @@
       </c>
     </row>
     <row r="10" spans="2:7">
-      <c r="C10" s="121" t="s">
+      <c r="C10" s="122" t="s">
         <v>917</v>
       </c>
-      <c r="D10" s="122"/>
-      <c r="E10" s="123"/>
+      <c r="D10" s="123"/>
+      <c r="E10" s="124"/>
       <c r="F10" t="s">
         <v>918</v>
       </c>
@@ -22651,9 +22800,9 @@
       </c>
     </row>
     <row r="11" spans="2:7" ht="15.75" thickBot="1">
-      <c r="C11" s="124"/>
-      <c r="D11" s="125"/>
-      <c r="E11" s="126"/>
+      <c r="C11" s="125"/>
+      <c r="D11" s="126"/>
+      <c r="E11" s="127"/>
       <c r="F11" t="s">
         <v>920</v>
       </c>
@@ -22674,129 +22823,84 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:L30"/>
+  <dimension ref="B2:E20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="2:12">
-      <c r="B2" s="6" t="s">
-        <v>974</v>
-      </c>
-    </row>
-    <row r="3" spans="2:12">
+    <row r="2" spans="2:5">
+      <c r="B2" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
       <c r="C3" t="s">
-        <v>976</v>
-      </c>
-    </row>
-    <row r="4" spans="2:12">
-      <c r="D4" t="s">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12">
-      <c r="C6" t="s">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12">
-      <c r="D7" t="s">
-        <v>977</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12">
-      <c r="D8" t="s">
-        <v>979</v>
-      </c>
-      <c r="L8" t="s">
-        <v>978</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12">
-      <c r="B10" t="s">
-        <v>981</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12">
-      <c r="C11" t="s">
-        <v>976</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12">
-      <c r="D12" t="s">
-        <v>984</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="C5" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="C7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="C8" t="s">
+        <v>1038</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5">
+      <c r="C10" s="17" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5">
+      <c r="C12" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="C13" s="17" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E13" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5">
       <c r="C14" t="s">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12">
-      <c r="D15" t="s">
-        <v>982</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12">
-      <c r="D16" t="s">
-        <v>983</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6">
-      <c r="D17" t="s">
-        <v>985</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6">
-      <c r="D19" t="s">
-        <v>986</v>
-      </c>
-      <c r="F19" t="s">
-        <v>987</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="D20" t="s">
-        <v>988</v>
-      </c>
-      <c r="F20" t="s">
-        <v>989</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6">
-      <c r="D21" t="s">
-        <v>990</v>
-      </c>
-      <c r="F21" t="s">
-        <v>991</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6">
-      <c r="B24" t="s">
-        <v>992</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6">
-      <c r="C25" t="s">
-        <v>976</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6">
-      <c r="D26" t="s">
-        <v>994</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6">
-      <c r="D27" t="s">
-        <v>993</v>
-      </c>
-    </row>
-    <row r="29" spans="2:6">
-      <c r="C29" t="s">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6">
-      <c r="D30" t="s">
-        <v>995</v>
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5">
+      <c r="C15" s="17" t="s">
+        <v>1033</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="134" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="C19" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="C20" t="s">
+        <v>1040</v>
       </c>
     </row>
   </sheetData>
@@ -22806,6 +22910,139 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:L30"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="2:12">
+      <c r="B2" s="6" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12">
+      <c r="C3" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12">
+      <c r="D4" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12">
+      <c r="C6" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12">
+      <c r="D7" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12">
+      <c r="D8" t="s">
+        <v>979</v>
+      </c>
+      <c r="L8" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12">
+      <c r="B10" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12">
+      <c r="C11" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12">
+      <c r="D12" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12">
+      <c r="C14" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12">
+      <c r="D15" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12">
+      <c r="D16" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6">
+      <c r="D17" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="D19" t="s">
+        <v>986</v>
+      </c>
+      <c r="F19" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="D20" t="s">
+        <v>988</v>
+      </c>
+      <c r="F20" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="D21" t="s">
+        <v>990</v>
+      </c>
+      <c r="F21" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="B24" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="C25" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6">
+      <c r="D26" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="D27" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6">
+      <c r="C29" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="D30" t="s">
+        <v>995</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:Q108"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -24610,7 +24847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:E27"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -24742,7 +24979,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:E37"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -24902,7 +25139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -25010,7 +25247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:F28"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -25143,162 +25380,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:F36"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="2" spans="2:4">
-      <c r="B2" s="6" t="s">
-        <v>809</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4">
-      <c r="C3" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4">
-      <c r="D4" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4">
-      <c r="C5" t="s">
-        <v>812</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4">
-      <c r="D6" t="s">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4">
-      <c r="D7" t="s">
-        <v>814</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4">
-      <c r="D8" t="s">
-        <v>815</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4">
-      <c r="D10" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4">
-      <c r="D12" t="s">
-        <v>817</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4">
-      <c r="D13" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4">
-      <c r="D14" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4">
-      <c r="D15" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4">
-      <c r="D16" t="s">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6">
-      <c r="D18" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6">
-      <c r="D20" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6">
-      <c r="C22" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6">
-      <c r="D23" t="s">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6">
-      <c r="D24" t="s">
-        <v>831</v>
-      </c>
-      <c r="F24" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="25" spans="2:6">
-      <c r="D25" t="s">
-        <v>830</v>
-      </c>
-      <c r="F25" t="s">
-        <v>827</v>
-      </c>
-    </row>
-    <row r="26" spans="2:6">
-      <c r="D26" t="s">
-        <v>829</v>
-      </c>
-      <c r="E26" t="s">
-        <v>828</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6">
-      <c r="D27" t="s">
-        <v>937</v>
-      </c>
-      <c r="F27" t="s">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6">
-      <c r="B30" t="s">
-        <v>938</v>
-      </c>
-    </row>
-    <row r="31" spans="2:6">
-      <c r="C31" t="s">
-        <v>941</v>
-      </c>
-    </row>
-    <row r="34" spans="3:3">
-      <c r="C34" t="s">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="35" spans="3:3">
-      <c r="C35" t="s">
-        <v>939</v>
-      </c>
-    </row>
-    <row r="36" spans="3:3">
-      <c r="C36" t="s">
-        <v>940</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:G113"/>
+  <dimension ref="B1:G128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="62.85546875" customWidth="1"/>
@@ -26432,7 +26516,7 @@
       <c r="B79" s="5">
         <v>17.5</v>
       </c>
-      <c r="C79" s="133" t="s">
+      <c r="C79" s="116" t="s">
         <v>454</v>
       </c>
       <c r="D79" s="6"/>
@@ -26552,195 +26636,144 @@
         <v>0</v>
       </c>
       <c r="E88" s="6"/>
-      <c r="F88" s="6"/>
+      <c r="F88" s="43" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="89" spans="2:6">
       <c r="B89" s="5">
         <v>21.1</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="D89" s="6"/>
+        <v>1027</v>
+      </c>
+      <c r="D89" s="51">
+        <v>0</v>
+      </c>
       <c r="E89" s="6"/>
-      <c r="F89" s="6"/>
-    </row>
-    <row r="90" spans="2:6" ht="30">
+      <c r="F89" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="90" spans="2:6">
       <c r="B90" s="5">
         <v>21.2</v>
       </c>
-      <c r="C90" s="7" t="s">
-        <v>468</v>
-      </c>
-      <c r="D90" s="6"/>
+      <c r="C90" s="6" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D90" s="51"/>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
     </row>
     <row r="91" spans="2:6">
-      <c r="B91" s="5" t="s">
-        <v>464</v>
+      <c r="B91" s="5">
+        <v>21.3</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>323</v>
-      </c>
-      <c r="D91" s="42">
-        <v>1</v>
-      </c>
-      <c r="E91" s="16" t="s">
-        <v>465</v>
-      </c>
-      <c r="F91" s="6" t="s">
-        <v>121</v>
-      </c>
+        <v>1043</v>
+      </c>
+      <c r="D91" s="51"/>
+      <c r="E91" s="6"/>
+      <c r="F91" s="6"/>
     </row>
     <row r="92" spans="2:6">
       <c r="B92" s="5">
-        <v>23.1</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>974</v>
-      </c>
-      <c r="D92" s="42">
-        <v>1</v>
-      </c>
-      <c r="E92" s="16"/>
-      <c r="F92" s="16" t="s">
-        <v>14</v>
-      </c>
+        <v>21.4</v>
+      </c>
+      <c r="C92" s="6"/>
+      <c r="D92" s="51"/>
+      <c r="E92" s="6"/>
+      <c r="F92" s="6"/>
     </row>
     <row r="93" spans="2:6">
       <c r="B93" s="5">
-        <v>23.2</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>981</v>
-      </c>
-      <c r="D93" s="42">
-        <v>1</v>
-      </c>
-      <c r="E93" s="16"/>
-      <c r="F93" s="16" t="s">
-        <v>14</v>
-      </c>
+        <v>21.5</v>
+      </c>
+      <c r="C93" s="6"/>
+      <c r="D93" s="51"/>
+      <c r="E93" s="6"/>
+      <c r="F93" s="6"/>
     </row>
     <row r="94" spans="2:6">
       <c r="B94" s="5">
-        <v>23.3</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>992</v>
-      </c>
-      <c r="D94" s="51">
-        <v>0.99</v>
-      </c>
-      <c r="E94" s="16"/>
-      <c r="F94" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="95" spans="2:6" ht="30">
-      <c r="B95" s="5" t="s">
-        <v>466</v>
-      </c>
-      <c r="C95" s="7" t="s">
-        <v>727</v>
-      </c>
-      <c r="D95" s="42">
-        <v>1</v>
-      </c>
-      <c r="E95" s="16" t="s">
-        <v>465</v>
-      </c>
-      <c r="F95" s="16"/>
+        <v>21.6</v>
+      </c>
+      <c r="C94" s="6"/>
+      <c r="D94" s="51"/>
+      <c r="E94" s="6"/>
+      <c r="F94" s="6"/>
+    </row>
+    <row r="95" spans="2:6">
+      <c r="B95" s="5">
+        <v>21.7</v>
+      </c>
+      <c r="C95" s="6"/>
+      <c r="D95" s="51"/>
+      <c r="E95" s="6"/>
+      <c r="F95" s="6"/>
     </row>
     <row r="96" spans="2:6">
       <c r="B96" s="5">
-        <v>24.1</v>
-      </c>
-      <c r="C96" s="7" t="s">
-        <v>728</v>
-      </c>
-      <c r="D96" s="42">
-        <v>1</v>
-      </c>
-      <c r="E96" s="16"/>
-      <c r="F96" s="16" t="s">
-        <v>14</v>
-      </c>
+        <v>21.8</v>
+      </c>
+      <c r="C96" s="6"/>
+      <c r="D96" s="51"/>
+      <c r="E96" s="6"/>
+      <c r="F96" s="6"/>
     </row>
     <row r="97" spans="2:7">
       <c r="B97" s="5">
-        <v>24.2</v>
-      </c>
-      <c r="C97" s="7" t="s">
-        <v>772</v>
-      </c>
-      <c r="D97" s="42">
+        <v>21.9</v>
+      </c>
+      <c r="C97" s="6"/>
+      <c r="D97" s="51"/>
+      <c r="E97" s="6"/>
+      <c r="F97" s="6"/>
+    </row>
+    <row r="98" spans="2:7">
+      <c r="B98" s="52" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C98" s="6"/>
+      <c r="D98" s="51"/>
+      <c r="E98" s="6"/>
+      <c r="F98" s="6"/>
+    </row>
+    <row r="99" spans="2:7">
+      <c r="B99" s="52" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="D99" s="6"/>
+      <c r="E99" s="6"/>
+      <c r="F99" s="6"/>
+    </row>
+    <row r="100" spans="2:7" ht="30">
+      <c r="B100" s="52" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D100" s="6"/>
+      <c r="E100" s="6"/>
+      <c r="F100" s="6"/>
+    </row>
+    <row r="101" spans="2:7">
+      <c r="B101" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="D101" s="42">
         <v>1</v>
       </c>
-      <c r="E97" s="16"/>
-      <c r="F97" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="G97" s="48"/>
-    </row>
-    <row r="98" spans="2:7">
-      <c r="B98" s="5" t="s">
-        <v>473</v>
-      </c>
-      <c r="C98" s="6" t="s">
-        <v>935</v>
-      </c>
-      <c r="D98" s="42">
-        <v>1</v>
-      </c>
-      <c r="E98" s="16"/>
-      <c r="F98" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="99" spans="2:7">
-      <c r="B99" s="5" t="s">
-        <v>475</v>
-      </c>
-      <c r="C99" s="6" t="s">
-        <v>477</v>
-      </c>
-      <c r="D99" s="42">
-        <v>1</v>
-      </c>
-      <c r="E99" s="16"/>
-      <c r="F99" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="100" spans="2:7">
-      <c r="B100" s="5">
-        <v>26.1</v>
-      </c>
-      <c r="C100" s="6" t="s">
-        <v>942</v>
-      </c>
-      <c r="D100" s="42">
-        <v>1</v>
-      </c>
-      <c r="E100" s="16"/>
-      <c r="F100" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="101" spans="2:7" ht="45">
-      <c r="B101" s="5" t="s">
-        <v>483</v>
-      </c>
-      <c r="C101" s="79" t="s">
-        <v>998</v>
-      </c>
-      <c r="D101" s="51">
-        <v>0.5</v>
-      </c>
       <c r="E101" s="16" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="F101" s="6" t="s">
         <v>121</v>
@@ -26748,13 +26781,13 @@
     </row>
     <row r="102" spans="2:7">
       <c r="B102" s="5">
-        <v>27.1</v>
-      </c>
-      <c r="C102" s="79" t="s">
-        <v>996</v>
-      </c>
-      <c r="D102" s="51">
-        <v>0.99</v>
+        <v>23.1</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>974</v>
+      </c>
+      <c r="D102" s="42">
+        <v>1</v>
       </c>
       <c r="E102" s="16"/>
       <c r="F102" s="16" t="s">
@@ -26763,55 +26796,55 @@
     </row>
     <row r="103" spans="2:7">
       <c r="B103" s="5">
-        <v>27.2</v>
-      </c>
-      <c r="C103" s="79" t="s">
-        <v>997</v>
-      </c>
-      <c r="D103" s="51">
+        <v>23.2</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>981</v>
+      </c>
+      <c r="D103" s="42">
+        <v>1</v>
+      </c>
+      <c r="E103" s="16"/>
+      <c r="F103" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="104" spans="2:7">
+      <c r="B104" s="5">
+        <v>23.3</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>992</v>
+      </c>
+      <c r="D104" s="51">
         <v>0.99</v>
-      </c>
-      <c r="E103" s="16"/>
-      <c r="F103" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="104" spans="2:7" ht="30">
-      <c r="B104" s="5" t="s">
-        <v>484</v>
-      </c>
-      <c r="C104" s="7" t="s">
-        <v>943</v>
-      </c>
-      <c r="D104" s="42">
-        <v>1</v>
       </c>
       <c r="E104" s="16"/>
       <c r="F104" s="16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="105" spans="2:7">
+    <row r="105" spans="2:7" ht="30">
       <c r="B105" s="5" t="s">
-        <v>485</v>
-      </c>
-      <c r="C105" s="6" t="s">
-        <v>809</v>
+        <v>466</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>727</v>
       </c>
       <c r="D105" s="42">
         <v>1</v>
       </c>
-      <c r="E105" s="16"/>
-      <c r="F105" s="16" t="s">
-        <v>14</v>
-      </c>
+      <c r="E105" s="16" t="s">
+        <v>465</v>
+      </c>
+      <c r="F105" s="16"/>
     </row>
     <row r="106" spans="2:7">
       <c r="B106" s="5">
-        <v>29.1</v>
-      </c>
-      <c r="C106" s="6" t="s">
-        <v>936</v>
+        <v>24.1</v>
+      </c>
+      <c r="C106" s="7" t="s">
+        <v>728</v>
       </c>
       <c r="D106" s="42">
         <v>1</v>
@@ -26822,11 +26855,11 @@
       </c>
     </row>
     <row r="107" spans="2:7">
-      <c r="B107" s="5" t="s">
-        <v>486</v>
+      <c r="B107" s="5">
+        <v>24.2</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>806</v>
+        <v>772</v>
       </c>
       <c r="D107" s="42">
         <v>1</v>
@@ -26835,13 +26868,14 @@
       <c r="F107" s="16" t="s">
         <v>14</v>
       </c>
+      <c r="G107" s="48"/>
     </row>
     <row r="108" spans="2:7">
-      <c r="B108" s="5">
-        <v>30.1</v>
-      </c>
-      <c r="C108" s="7" t="s">
-        <v>803</v>
+      <c r="B108" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>935</v>
       </c>
       <c r="D108" s="42">
         <v>1</v>
@@ -26852,11 +26886,11 @@
       </c>
     </row>
     <row r="109" spans="2:7">
-      <c r="B109" s="5">
-        <v>30.2</v>
-      </c>
-      <c r="C109" s="7" t="s">
-        <v>804</v>
+      <c r="B109" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>477</v>
       </c>
       <c r="D109" s="42">
         <v>1</v>
@@ -26865,14 +26899,13 @@
       <c r="F109" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G109" s="48"/>
     </row>
     <row r="110" spans="2:7">
       <c r="B110" s="5">
-        <v>30.3</v>
-      </c>
-      <c r="C110" s="7" t="s">
-        <v>805</v>
+        <v>26.1</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>942</v>
       </c>
       <c r="D110" s="42">
         <v>1</v>
@@ -26882,48 +26915,246 @@
         <v>14</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="30">
+    <row r="111" spans="2:7" ht="45">
       <c r="B111" s="5" t="s">
-        <v>487</v>
-      </c>
-      <c r="C111" s="7" t="s">
-        <v>474</v>
+        <v>483</v>
+      </c>
+      <c r="C111" s="79" t="s">
+        <v>998</v>
       </c>
       <c r="D111" s="51">
-        <v>0.05</v>
-      </c>
-      <c r="E111" s="16"/>
-      <c r="F111" s="16" t="s">
-        <v>14</v>
+        <v>0.5</v>
+      </c>
+      <c r="E111" s="16" t="s">
+        <v>480</v>
+      </c>
+      <c r="F111" s="6" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="112" spans="2:7">
-      <c r="B112" s="5" t="s">
-        <v>773</v>
-      </c>
-      <c r="C112" s="7" t="s">
-        <v>774</v>
-      </c>
-      <c r="D112" s="42">
-        <v>1</v>
+      <c r="B112" s="5">
+        <v>27.1</v>
+      </c>
+      <c r="C112" s="79" t="s">
+        <v>996</v>
+      </c>
+      <c r="D112" s="51">
+        <v>0.99</v>
       </c>
       <c r="E112" s="16"/>
       <c r="F112" s="16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="113" spans="2:6">
-      <c r="B113" s="77" t="s">
+    <row r="113" spans="2:7">
+      <c r="B113" s="5">
+        <v>27.2</v>
+      </c>
+      <c r="C113" s="79" t="s">
+        <v>997</v>
+      </c>
+      <c r="D113" s="51">
+        <v>0.99</v>
+      </c>
+      <c r="E113" s="16"/>
+      <c r="F113" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="114" spans="2:7" ht="30">
+      <c r="B114" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>943</v>
+      </c>
+      <c r="D114" s="42">
+        <v>1</v>
+      </c>
+      <c r="E114" s="16"/>
+      <c r="F114" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="115" spans="2:7">
+      <c r="B115" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="C115" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="D115" s="42">
+        <v>1</v>
+      </c>
+      <c r="E115" s="16"/>
+      <c r="F115" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="116" spans="2:7">
+      <c r="B116" s="5">
+        <v>29.1</v>
+      </c>
+      <c r="C116" s="6" t="s">
+        <v>936</v>
+      </c>
+      <c r="D116" s="42">
+        <v>1</v>
+      </c>
+      <c r="E116" s="16"/>
+      <c r="F116" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="117" spans="2:7">
+      <c r="B117" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>806</v>
+      </c>
+      <c r="D117" s="42">
+        <v>1</v>
+      </c>
+      <c r="E117" s="16"/>
+      <c r="F117" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="118" spans="2:7">
+      <c r="B118" s="5">
+        <v>30.1</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="D118" s="42">
+        <v>1</v>
+      </c>
+      <c r="E118" s="16"/>
+      <c r="F118" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="119" spans="2:7">
+      <c r="B119" s="5">
+        <v>30.2</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="D119" s="42">
+        <v>1</v>
+      </c>
+      <c r="E119" s="16"/>
+      <c r="F119" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G119" s="48"/>
+    </row>
+    <row r="120" spans="2:7">
+      <c r="B120" s="5">
+        <v>30.3</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>805</v>
+      </c>
+      <c r="D120" s="42">
+        <v>1</v>
+      </c>
+      <c r="E120" s="16"/>
+      <c r="F120" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121" spans="2:7" ht="30">
+      <c r="B121" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="C121" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="D121" s="51">
+        <v>0.05</v>
+      </c>
+      <c r="E121" s="16"/>
+      <c r="F121" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="122" spans="2:7">
+      <c r="B122" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="D122" s="42">
+        <v>1</v>
+      </c>
+      <c r="E122" s="16"/>
+      <c r="F122" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="123" spans="2:7">
+      <c r="B123" s="5" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C123" s="7" t="s">
+        <v>1021</v>
+      </c>
+      <c r="D123" s="42"/>
+      <c r="E123" s="16"/>
+      <c r="F123" s="16"/>
+    </row>
+    <row r="124" spans="2:7">
+      <c r="B124" s="5"/>
+      <c r="C124" s="7" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D124" s="42"/>
+      <c r="E124" s="16"/>
+      <c r="F124" s="16"/>
+    </row>
+    <row r="125" spans="2:7">
+      <c r="B125" s="5"/>
+      <c r="C125" s="7" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D125" s="42"/>
+      <c r="E125" s="16"/>
+      <c r="F125" s="16"/>
+    </row>
+    <row r="126" spans="2:7">
+      <c r="B126" s="5"/>
+      <c r="C126" s="7" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D126" s="42"/>
+      <c r="E126" s="16"/>
+      <c r="F126" s="16"/>
+    </row>
+    <row r="127" spans="2:7">
+      <c r="B127" s="5"/>
+      <c r="C127" s="7"/>
+      <c r="D127" s="42"/>
+      <c r="E127" s="16"/>
+      <c r="F127" s="16"/>
+    </row>
+    <row r="128" spans="2:7">
+      <c r="B128" s="77" t="s">
         <v>471</v>
       </c>
-      <c r="C113" s="57" t="s">
+      <c r="C128" s="57" t="s">
         <v>470</v>
       </c>
-      <c r="D113" s="1"/>
-      <c r="E113" s="49" t="s">
+      <c r="D128" s="1"/>
+      <c r="E128" s="49" t="s">
         <v>469</v>
       </c>
-      <c r="F113" s="1"/>
+      <c r="F128" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -26975,9 +27206,9 @@
     <hyperlink ref="F62" location="'#14'!B2" display="Link"/>
     <hyperlink ref="E64" r:id="rId7"/>
     <hyperlink ref="E77" r:id="rId8"/>
-    <hyperlink ref="E91" r:id="rId9"/>
-    <hyperlink ref="E95" r:id="rId10"/>
-    <hyperlink ref="E113" r:id="rId11"/>
+    <hyperlink ref="E101" r:id="rId9"/>
+    <hyperlink ref="E105" r:id="rId10"/>
+    <hyperlink ref="E128" r:id="rId11"/>
     <hyperlink ref="F49" location="'#9'!B2" display="Link"/>
     <hyperlink ref="F60" location="'#12'!B2" display="Link"/>
     <hyperlink ref="F65" location="'#16'!B2" display="Link"/>
@@ -26990,19 +27221,19 @@
     <hyperlink ref="F63" location="'#15'!B2" display="Link"/>
     <hyperlink ref="F70" location="'#16'!B89" display="Link"/>
     <hyperlink ref="F71" location="'#16'!B10" display="Link"/>
-    <hyperlink ref="F111" location="'#31'!B2" display="Link"/>
-    <hyperlink ref="F96" location="'#24'!B2" display="Link"/>
-    <hyperlink ref="F97" location="'#24'!B2" display="Link"/>
-    <hyperlink ref="F97:G97" location="'#24'!B26" display="Link"/>
-    <hyperlink ref="F98" location="'#25'!B2" display="Link"/>
+    <hyperlink ref="F121" location="'#31'!B2" display="Link"/>
+    <hyperlink ref="F106" location="'#24'!B2" display="Link"/>
+    <hyperlink ref="F107" location="'#24'!B2" display="Link"/>
+    <hyperlink ref="F107:G107" location="'#24'!B26" display="Link"/>
+    <hyperlink ref="F108" location="'#25'!B2" display="Link"/>
     <hyperlink ref="F86" location="'#19'!B2" display="Link"/>
-    <hyperlink ref="F108" location="'#30'!B8" display="Link"/>
-    <hyperlink ref="F105" location="'#29'!B2" display="Link"/>
-    <hyperlink ref="F112" location="'#32'!B2" display="Link"/>
-    <hyperlink ref="F107" location="'#30'!B2" display="Link"/>
-    <hyperlink ref="F109" location="'#30'!B8" display="Link"/>
-    <hyperlink ref="F109:G109" location="'#30'!B24" display="Link"/>
-    <hyperlink ref="F110" location="'#30'!B35" display="Link"/>
+    <hyperlink ref="F118" location="'#30'!B8" display="Link"/>
+    <hyperlink ref="F115" location="'#29'!B2" display="Link"/>
+    <hyperlink ref="F122" location="'#32'!B2" display="Link"/>
+    <hyperlink ref="F117" location="'#30'!B2" display="Link"/>
+    <hyperlink ref="F119" location="'#30'!B8" display="Link"/>
+    <hyperlink ref="F119:G119" location="'#30'!B24" display="Link"/>
+    <hyperlink ref="F120" location="'#30'!B35" display="Link"/>
     <hyperlink ref="F51" location="'#11'!B2" display="Link"/>
     <hyperlink ref="F52" location="'#11'!B4" display="Link"/>
     <hyperlink ref="F53" location="'#11'!B21" display="Link"/>
@@ -27011,14 +27242,16 @@
     <hyperlink ref="F28" location="'#4'!B35" display="Link"/>
     <hyperlink ref="F29" location="'#4'!B43" display="Link"/>
     <hyperlink ref="F87" location="'#20'!B2" display="Link"/>
-    <hyperlink ref="F99" location="'#26'!B2" display="Link"/>
-    <hyperlink ref="F106" location="'#29'!B30" display="Link"/>
-    <hyperlink ref="F104" location="'#28'!B17" display="Link"/>
-    <hyperlink ref="F100" location="'#26'!B22" display="Link"/>
-    <hyperlink ref="F92" location="'#23'!B2" display="Link"/>
-    <hyperlink ref="F93" location="'#23'!B10" display="Link"/>
-    <hyperlink ref="F94" location="'#23'!B24" display="Link"/>
-    <hyperlink ref="F102" location="'#27'!B2" display="Link"/>
+    <hyperlink ref="F109" location="'#26'!B2" display="Link"/>
+    <hyperlink ref="F116" location="'#29'!B30" display="Link"/>
+    <hyperlink ref="F114" location="'#28'!B17" display="Link"/>
+    <hyperlink ref="F110" location="'#26'!B22" display="Link"/>
+    <hyperlink ref="F102" location="'#23'!B2" display="Link"/>
+    <hyperlink ref="F103" location="'#23'!B10" display="Link"/>
+    <hyperlink ref="F104" location="'#23'!B24" display="Link"/>
+    <hyperlink ref="F112" location="'#27'!B2" display="Link"/>
+    <hyperlink ref="F113" location="'#27'!B18" display="Link"/>
+    <hyperlink ref="F89" location="'#21'!B2" display="Link"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId12"/>
@@ -27026,6 +27259,159 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:F36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="B2" s="6" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4">
+      <c r="C3" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4">
+      <c r="D4" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="C5" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="D6" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="D7" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="D8" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4">
+      <c r="D10" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4">
+      <c r="D12" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="D13" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="D14" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4">
+      <c r="D15" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="D16" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="D18" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="D20" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="C22" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="D23" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="D24" t="s">
+        <v>831</v>
+      </c>
+      <c r="F24" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="D25" t="s">
+        <v>830</v>
+      </c>
+      <c r="F25" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6">
+      <c r="D26" t="s">
+        <v>829</v>
+      </c>
+      <c r="E26" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="D27" t="s">
+        <v>937</v>
+      </c>
+      <c r="F27" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="B30" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6">
+      <c r="C31" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3">
+      <c r="C35" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3">
+      <c r="C36" t="s">
+        <v>940</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:B39"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -27182,7 +27568,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:O20"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -27244,21 +27630,21 @@
       <c r="D16" t="s">
         <v>712</v>
       </c>
-      <c r="I16" s="127" t="s">
+      <c r="I16" s="128" t="s">
         <v>716</v>
       </c>
-      <c r="J16" s="128"/>
+      <c r="J16" s="129"/>
     </row>
     <row r="17" spans="3:10" ht="15" customHeight="1">
-      <c r="I17" s="129"/>
-      <c r="J17" s="130"/>
+      <c r="I17" s="130"/>
+      <c r="J17" s="131"/>
     </row>
     <row r="18" spans="3:10">
       <c r="D18" t="s">
         <v>713</v>
       </c>
-      <c r="I18" s="131"/>
-      <c r="J18" s="132"/>
+      <c r="I18" s="132"/>
+      <c r="J18" s="133"/>
     </row>
     <row r="19" spans="3:10">
       <c r="C19" t="s">
@@ -27279,7 +27665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:K18"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -27677,7 +28063,7 @@
       <c r="D12" s="11"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1">
-      <c r="C13" s="116" t="s">
+      <c r="C13" s="117" t="s">
         <v>78</v>
       </c>
       <c r="D13" s="26" t="s">
@@ -27694,7 +28080,7 @@
       <c r="I13" s="25"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" thickBot="1">
-      <c r="C14" s="117"/>
+      <c r="C14" s="118"/>
       <c r="D14" s="23" t="s">
         <v>65</v>
       </c>
@@ -27710,7 +28096,7 @@
       <c r="J14" s="25"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="C15" s="117"/>
+      <c r="C15" s="118"/>
       <c r="D15" s="26" t="s">
         <v>66</v>
       </c>
@@ -27725,7 +28111,7 @@
       <c r="I15" s="28"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="C16" s="117"/>
+      <c r="C16" s="118"/>
       <c r="D16" s="29"/>
       <c r="E16" s="30" t="s">
         <v>74</v>
@@ -27736,7 +28122,7 @@
       <c r="I16" s="31"/>
     </row>
     <row r="17" spans="3:12" ht="15.75" thickBot="1">
-      <c r="C17" s="118"/>
+      <c r="C17" s="119"/>
       <c r="D17" s="32"/>
       <c r="E17" s="33" t="s">
         <v>75</v>
@@ -27767,7 +28153,7 @@
       <c r="L18" s="25"/>
     </row>
     <row r="19" spans="3:12" ht="15.75" thickBot="1">
-      <c r="C19" s="116" t="s">
+      <c r="C19" s="117" t="s">
         <v>78</v>
       </c>
       <c r="D19" s="23" t="s">
@@ -27778,7 +28164,7 @@
       </c>
     </row>
     <row r="20" spans="3:12">
-      <c r="C20" s="117"/>
+      <c r="C20" s="118"/>
       <c r="D20" s="26" t="s">
         <v>82</v>
       </c>
@@ -27787,7 +28173,7 @@
       </c>
     </row>
     <row r="21" spans="3:12" ht="15.75" thickBot="1">
-      <c r="C21" s="118"/>
+      <c r="C21" s="119"/>
       <c r="D21" s="32"/>
       <c r="E21" s="40" t="s">
         <v>84</v>

</xml_diff>